<commit_message>
Teklif ve sözleşme şablon çıktısını güncelle
Excel ana şablonu yeni nihai düzenle uyumlu hale getirildi; Times New Roman kullanımı, büyük harfli tablo başlıkları, alt banner, ödeme/teslimat, banka ve imza blokları export akışına bağlandı.

YEKÜN İCMAALLERİ alanı artık sabit boş satırlar basmak yerine yalnızca satış veya masraf oluşan ürün gruplarını dinamik gösteriyor. Eski verilerdeki ÇELİK KAPI gibi metinsel grup anahtarları kanonik grup anahtarlarına çevrilerek toplamlar doğru gruba yazılıyor.

Hizmetler & montaj masrafları teklif/sözleşme oluşturma ekranında ayrı sekmeye taşındı; seçilen ürün gruplarına göre masraf satırları senkronize ediliyor ve Excel çıktısında ürün kodu yerine ürün kategori bazlı gösteriliyor.

Yeni şirket oluşturma doğrulama mesajları iyileştirildi, sektör/grup uzunluğu daha anlaşılır hale getirildi ve teklif formundaki Zod kayıt tanımı düzeltilerek kaydetme hatası giderildi.

Doğrulama: backend py_compile ve frontend npm run build başarılı.
</commit_message>
<xml_diff>
--- a/backend/crm/assets/contract-templates/MASTER/SELLER_MASTER_TEMPLATE.xlsx
+++ b/backend/crm/assets/contract-templates/MASTER/SELLER_MASTER_TEMPLATE.xlsx
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;₺&quot;* #,##0.00_-;\-&quot;₺&quot;* #,##0.00_-;_-&quot;₺&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -151,6 +151,29 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <charset val="162"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color rgb="FF000066"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <charset val="162"/>
+      <family val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <charset val="162"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color rgb="FF203864"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -305,7 +328,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -384,6 +407,33 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,74 +882,46 @@
           <t>{saticiLogo}</t>
         </is>
       </c>
-      <c r="C2" s="26" t="n"/>
-      <c r="D2" s="26" t="n"/>
-      <c r="E2" s="26" t="n"/>
       <c r="F2" s="26" t="n"/>
       <c r="G2" s="26" t="n"/>
       <c r="H2" s="26" t="n"/>
       <c r="I2" s="26" t="n"/>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="38" t="inlineStr">
         <is>
           <t>{seciliSatici.resmiUnvan}</t>
         </is>
       </c>
-      <c r="K2" s="26" t="n"/>
-      <c r="L2" s="26" t="n"/>
-      <c r="M2" s="26" t="n"/>
     </row>
     <row r="3" ht="23" customHeight="1" s="1">
       <c r="A3" s="26" t="n"/>
-      <c r="B3" s="26" t="n"/>
-      <c r="C3" s="26" t="n"/>
-      <c r="D3" s="26" t="n"/>
-      <c r="E3" s="26" t="n"/>
       <c r="F3" s="26" t="n"/>
       <c r="G3" s="26" t="n"/>
       <c r="H3" s="26" t="n"/>
       <c r="I3" s="26" t="n"/>
-      <c r="J3" s="26" t="n"/>
-      <c r="K3" s="26" t="n"/>
-      <c r="L3" s="26" t="n"/>
-      <c r="M3" s="26" t="n"/>
     </row>
     <row r="4" ht="23" customHeight="1" s="1">
       <c r="A4" s="26" t="n"/>
-      <c r="B4" s="26" t="n"/>
-      <c r="C4" s="26" t="n"/>
-      <c r="D4" s="26" t="n"/>
-      <c r="E4" s="26" t="n"/>
       <c r="F4" s="26" t="n"/>
       <c r="G4" s="26" t="n"/>
       <c r="H4" s="26" t="n"/>
       <c r="I4" s="26" t="n"/>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="38" t="inlineStr">
         <is>
           <t>{seciliSatici.kisaAd}</t>
         </is>
       </c>
-      <c r="K4" s="26" t="n"/>
-      <c r="L4" s="26" t="n"/>
-      <c r="M4" s="26" t="n"/>
     </row>
     <row r="5" ht="23" customHeight="1" s="1">
       <c r="A5" s="26" t="n"/>
-      <c r="B5" s="26" t="n"/>
-      <c r="C5" s="26" t="n"/>
-      <c r="D5" s="26" t="n"/>
-      <c r="E5" s="26" t="n"/>
       <c r="F5" s="26" t="n"/>
       <c r="G5" s="26" t="n"/>
       <c r="H5" s="26" t="n"/>
       <c r="I5" s="26" t="n"/>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="38" t="inlineStr">
         <is>
           <t>{seciliSatici.email} / {seciliSatici.telefon}</t>
         </is>
       </c>
-      <c r="K5" s="26" t="n"/>
-      <c r="L5" s="26" t="n"/>
-      <c r="M5" s="26" t="n"/>
     </row>
     <row r="6" ht="23" customHeight="1" s="1">
       <c r="A6" s="26" t="n"/>
@@ -916,24 +938,24 @@
       <c r="L6" s="26" t="n"/>
       <c r="M6" s="26" t="n"/>
     </row>
-    <row r="7" ht="23" customHeight="1" s="1">
+    <row r="7" ht="26" customHeight="1" s="1">
       <c r="A7" s="26" t="n"/>
       <c r="B7" s="17" t="inlineStr">
         <is>
           <t>{belgeTuru}</t>
         </is>
       </c>
-      <c r="C7" s="27" t="n"/>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="27" t="n"/>
-      <c r="I7" s="27" t="n"/>
-      <c r="J7" s="27" t="n"/>
-      <c r="K7" s="27" t="n"/>
-      <c r="L7" s="27" t="n"/>
-      <c r="M7" s="28" t="n"/>
+      <c r="C7" s="39" t="n"/>
+      <c r="D7" s="39" t="n"/>
+      <c r="E7" s="39" t="n"/>
+      <c r="F7" s="39" t="n"/>
+      <c r="G7" s="39" t="n"/>
+      <c r="H7" s="39" t="n"/>
+      <c r="I7" s="39" t="n"/>
+      <c r="J7" s="39" t="n"/>
+      <c r="K7" s="39" t="n"/>
+      <c r="L7" s="39" t="n"/>
+      <c r="M7" s="40" t="n"/>
     </row>
     <row r="8" ht="23" customHeight="1" s="1">
       <c r="A8" s="26" t="n"/>
@@ -946,13 +968,13 @@
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="9" t="n"/>
-      <c r="K8" s="10" t="inlineStr">
+      <c r="K8" s="41" t="inlineStr">
         <is>
           <t>TARİH</t>
         </is>
       </c>
-      <c r="L8" s="28" t="n"/>
-      <c r="M8" s="10" t="inlineStr">
+      <c r="L8" s="40" t="n"/>
+      <c r="M8" s="41" t="inlineStr">
         <is>
           <t>{olusturmaTarihi}</t>
         </is>
@@ -976,112 +998,107 @@
           <t>SATIŞI YAPAN FİRMA</t>
         </is>
       </c>
-      <c r="C9" s="27" t="n"/>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="27" t="n"/>
-      <c r="I9" s="27" t="n"/>
-      <c r="J9" s="27" t="n"/>
-      <c r="K9" s="27" t="n"/>
-      <c r="L9" s="27" t="n"/>
-      <c r="M9" s="28" t="n"/>
+      <c r="C9" s="39" t="n"/>
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39" t="n"/>
+      <c r="G9" s="39" t="n"/>
+      <c r="H9" s="39" t="n"/>
+      <c r="I9" s="39" t="n"/>
+      <c r="J9" s="39" t="n"/>
+      <c r="K9" s="39" t="n"/>
+      <c r="L9" s="39" t="n"/>
+      <c r="M9" s="40" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1" s="1">
-      <c r="A10" s="26" t="n"/>
       <c r="B10" s="22" t="inlineStr">
         <is>
           <t>ÜNVAN</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n"/>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="C10" s="40" t="n"/>
+      <c r="D10" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.resmiUnvan}</t>
         </is>
       </c>
-      <c r="E10" s="27" t="n"/>
-      <c r="F10" s="27" t="n"/>
-      <c r="G10" s="27" t="n"/>
-      <c r="H10" s="27" t="n"/>
-      <c r="I10" s="27" t="n"/>
-      <c r="J10" s="27" t="n"/>
-      <c r="K10" s="27" t="n"/>
-      <c r="L10" s="27" t="n"/>
-      <c r="M10" s="28" t="n"/>
+      <c r="E10" s="39" t="n"/>
+      <c r="F10" s="39" t="n"/>
+      <c r="G10" s="39" t="n"/>
+      <c r="H10" s="39" t="n"/>
+      <c r="I10" s="39" t="n"/>
+      <c r="J10" s="39" t="n"/>
+      <c r="K10" s="39" t="n"/>
+      <c r="L10" s="39" t="n"/>
+      <c r="M10" s="40" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1" s="1">
-      <c r="A11" s="26" t="n"/>
       <c r="B11" s="22" t="inlineStr">
         <is>
           <t>VERGİ DAİRESİ / NO</t>
         </is>
       </c>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.vergiDairesi} / {seciliSatici.vergiNo}</t>
         </is>
       </c>
-      <c r="E11" s="27" t="n"/>
-      <c r="F11" s="27" t="n"/>
-      <c r="G11" s="27" t="n"/>
-      <c r="H11" s="27" t="n"/>
-      <c r="I11" s="27" t="n"/>
-      <c r="J11" s="27" t="n"/>
-      <c r="K11" s="27" t="n"/>
-      <c r="L11" s="27" t="n"/>
-      <c r="M11" s="28" t="n"/>
+      <c r="E11" s="39" t="n"/>
+      <c r="F11" s="39" t="n"/>
+      <c r="G11" s="39" t="n"/>
+      <c r="H11" s="39" t="n"/>
+      <c r="I11" s="39" t="n"/>
+      <c r="J11" s="39" t="n"/>
+      <c r="K11" s="39" t="n"/>
+      <c r="L11" s="39" t="n"/>
+      <c r="M11" s="40" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1" s="1">
-      <c r="A12" s="26" t="n"/>
       <c r="B12" s="22" t="inlineStr">
         <is>
           <t>ADRES</t>
         </is>
       </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="C12" s="40" t="n"/>
+      <c r="D12" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.adres}</t>
         </is>
       </c>
-      <c r="E12" s="27" t="n"/>
-      <c r="F12" s="27" t="n"/>
-      <c r="G12" s="27" t="n"/>
-      <c r="H12" s="27" t="n"/>
-      <c r="I12" s="27" t="n"/>
-      <c r="J12" s="27" t="n"/>
-      <c r="K12" s="27" t="n"/>
-      <c r="L12" s="27" t="n"/>
-      <c r="M12" s="28" t="n"/>
+      <c r="E12" s="39" t="n"/>
+      <c r="F12" s="39" t="n"/>
+      <c r="G12" s="39" t="n"/>
+      <c r="H12" s="39" t="n"/>
+      <c r="I12" s="39" t="n"/>
+      <c r="J12" s="39" t="n"/>
+      <c r="K12" s="39" t="n"/>
+      <c r="L12" s="39" t="n"/>
+      <c r="M12" s="40" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1" s="1">
-      <c r="A13" s="26" t="n"/>
       <c r="B13" s="22" t="inlineStr">
         <is>
           <t>TELEFON / E-POSTA</t>
         </is>
       </c>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="C13" s="40" t="n"/>
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.telefon} / {seciliSatici.email}</t>
         </is>
       </c>
-      <c r="E13" s="27" t="n"/>
-      <c r="F13" s="27" t="n"/>
-      <c r="G13" s="27" t="n"/>
-      <c r="H13" s="27" t="n"/>
-      <c r="I13" s="27" t="n"/>
-      <c r="J13" s="27" t="n"/>
-      <c r="K13" s="27" t="n"/>
-      <c r="L13" s="27" t="n"/>
-      <c r="M13" s="28" t="n"/>
+      <c r="E13" s="39" t="n"/>
+      <c r="F13" s="39" t="n"/>
+      <c r="G13" s="39" t="n"/>
+      <c r="H13" s="39" t="n"/>
+      <c r="I13" s="39" t="n"/>
+      <c r="J13" s="39" t="n"/>
+      <c r="K13" s="39" t="n"/>
+      <c r="L13" s="39" t="n"/>
+      <c r="M13" s="40" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1" s="1">
-      <c r="A14" s="26" t="n"/>
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="9" t="n"/>
@@ -1096,141 +1113,134 @@
       <c r="M14" s="9" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1" s="1">
-      <c r="A15" s="26" t="n"/>
       <c r="B15" s="15" t="inlineStr">
         <is>
           <t>ALICI BİLGİLERİ</t>
         </is>
       </c>
-      <c r="C15" s="27" t="n"/>
-      <c r="D15" s="27" t="n"/>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="27" t="n"/>
-      <c r="H15" s="27" t="n"/>
-      <c r="I15" s="27" t="n"/>
-      <c r="J15" s="27" t="n"/>
-      <c r="K15" s="27" t="n"/>
-      <c r="L15" s="27" t="n"/>
-      <c r="M15" s="28" t="n"/>
+      <c r="C15" s="39" t="n"/>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="39" t="n"/>
+      <c r="F15" s="39" t="n"/>
+      <c r="G15" s="39" t="n"/>
+      <c r="H15" s="39" t="n"/>
+      <c r="I15" s="39" t="n"/>
+      <c r="J15" s="39" t="n"/>
+      <c r="K15" s="39" t="n"/>
+      <c r="L15" s="39" t="n"/>
+      <c r="M15" s="40" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1" s="1">
-      <c r="A16" s="26" t="n"/>
       <c r="B16" s="22" t="inlineStr">
         <is>
           <t>CARİ ÜNVANI</t>
         </is>
       </c>
-      <c r="C16" s="28" t="n"/>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="C16" s="40" t="n"/>
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>{cariUnvani}</t>
         </is>
       </c>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="27" t="n"/>
-      <c r="G16" s="27" t="n"/>
-      <c r="H16" s="27" t="n"/>
-      <c r="I16" s="27" t="n"/>
-      <c r="J16" s="27" t="n"/>
-      <c r="K16" s="27" t="n"/>
-      <c r="L16" s="27" t="n"/>
-      <c r="M16" s="28" t="n"/>
+      <c r="E16" s="39" t="n"/>
+      <c r="F16" s="39" t="n"/>
+      <c r="G16" s="39" t="n"/>
+      <c r="H16" s="39" t="n"/>
+      <c r="I16" s="39" t="n"/>
+      <c r="J16" s="39" t="n"/>
+      <c r="K16" s="39" t="n"/>
+      <c r="L16" s="39" t="n"/>
+      <c r="M16" s="40" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1" s="1">
-      <c r="A17" s="26" t="n"/>
       <c r="B17" s="22" t="inlineStr">
         <is>
           <t>VERGİ DAİRESİ / NO</t>
         </is>
       </c>
-      <c r="C17" s="28" t="n"/>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="C17" s="40" t="n"/>
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>{vergiDairesi} / {vergiNo}</t>
         </is>
       </c>
-      <c r="E17" s="27" t="n"/>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
-      <c r="H17" s="27" t="n"/>
-      <c r="I17" s="27" t="n"/>
-      <c r="J17" s="27" t="n"/>
-      <c r="K17" s="27" t="n"/>
-      <c r="L17" s="27" t="n"/>
-      <c r="M17" s="28" t="n"/>
+      <c r="E17" s="39" t="n"/>
+      <c r="F17" s="39" t="n"/>
+      <c r="G17" s="39" t="n"/>
+      <c r="H17" s="39" t="n"/>
+      <c r="I17" s="39" t="n"/>
+      <c r="J17" s="39" t="n"/>
+      <c r="K17" s="39" t="n"/>
+      <c r="L17" s="39" t="n"/>
+      <c r="M17" s="40" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1" s="1">
-      <c r="A18" s="26" t="n"/>
       <c r="B18" s="22" t="inlineStr">
         <is>
           <t>ADRES</t>
         </is>
       </c>
-      <c r="C18" s="28" t="n"/>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="C18" s="40" t="n"/>
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>{adres}</t>
         </is>
       </c>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="27" t="n"/>
-      <c r="G18" s="27" t="n"/>
-      <c r="H18" s="27" t="n"/>
-      <c r="I18" s="27" t="n"/>
-      <c r="J18" s="27" t="n"/>
-      <c r="K18" s="27" t="n"/>
-      <c r="L18" s="27" t="n"/>
-      <c r="M18" s="28" t="n"/>
+      <c r="E18" s="39" t="n"/>
+      <c r="F18" s="39" t="n"/>
+      <c r="G18" s="39" t="n"/>
+      <c r="H18" s="39" t="n"/>
+      <c r="I18" s="39" t="n"/>
+      <c r="J18" s="39" t="n"/>
+      <c r="K18" s="39" t="n"/>
+      <c r="L18" s="39" t="n"/>
+      <c r="M18" s="40" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1" s="1">
-      <c r="A19" s="26" t="n"/>
       <c r="B19" s="22" t="inlineStr">
         <is>
           <t>YETKİLİ</t>
         </is>
       </c>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="C19" s="40" t="n"/>
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>{yetkili}</t>
         </is>
       </c>
-      <c r="E19" s="27" t="n"/>
-      <c r="F19" s="27" t="n"/>
-      <c r="G19" s="27" t="n"/>
-      <c r="H19" s="27" t="n"/>
-      <c r="I19" s="27" t="n"/>
-      <c r="J19" s="27" t="n"/>
-      <c r="K19" s="27" t="n"/>
-      <c r="L19" s="27" t="n"/>
-      <c r="M19" s="28" t="n"/>
+      <c r="E19" s="39" t="n"/>
+      <c r="F19" s="39" t="n"/>
+      <c r="G19" s="39" t="n"/>
+      <c r="H19" s="39" t="n"/>
+      <c r="I19" s="39" t="n"/>
+      <c r="J19" s="39" t="n"/>
+      <c r="K19" s="39" t="n"/>
+      <c r="L19" s="39" t="n"/>
+      <c r="M19" s="40" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1" s="1">
-      <c r="A20" s="26" t="n"/>
       <c r="B20" s="22" t="inlineStr">
         <is>
           <t>TELEFON / E-POSTA</t>
         </is>
       </c>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="C20" s="40" t="n"/>
+      <c r="D20" s="42" t="inlineStr">
         <is>
           <t>{telefon} / {email}</t>
         </is>
       </c>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="27" t="n"/>
-      <c r="G20" s="27" t="n"/>
-      <c r="H20" s="27" t="n"/>
-      <c r="I20" s="27" t="n"/>
-      <c r="J20" s="27" t="n"/>
-      <c r="K20" s="27" t="n"/>
-      <c r="L20" s="27" t="n"/>
-      <c r="M20" s="28" t="n"/>
+      <c r="E20" s="39" t="n"/>
+      <c r="F20" s="39" t="n"/>
+      <c r="G20" s="39" t="n"/>
+      <c r="H20" s="39" t="n"/>
+      <c r="I20" s="39" t="n"/>
+      <c r="J20" s="39" t="n"/>
+      <c r="K20" s="39" t="n"/>
+      <c r="L20" s="39" t="n"/>
+      <c r="M20" s="40" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1" s="1">
-      <c r="A21" s="26" t="n"/>
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="9" t="n"/>
       <c r="D21" s="9" t="n"/>
@@ -1245,115 +1255,110 @@
       <c r="M21" s="9" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1" s="1">
-      <c r="A22" s="26" t="n"/>
       <c r="B22" s="15" t="inlineStr">
         <is>
           <t>{belgeTuru} DETAYLARI</t>
         </is>
       </c>
-      <c r="C22" s="27" t="n"/>
-      <c r="D22" s="27" t="n"/>
-      <c r="E22" s="27" t="n"/>
-      <c r="F22" s="27" t="n"/>
-      <c r="G22" s="27" t="n"/>
-      <c r="H22" s="27" t="n"/>
-      <c r="I22" s="27" t="n"/>
-      <c r="J22" s="27" t="n"/>
-      <c r="K22" s="27" t="n"/>
-      <c r="L22" s="27" t="n"/>
-      <c r="M22" s="28" t="n"/>
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="39" t="n"/>
+      <c r="E22" s="39" t="n"/>
+      <c r="F22" s="39" t="n"/>
+      <c r="G22" s="39" t="n"/>
+      <c r="H22" s="39" t="n"/>
+      <c r="I22" s="39" t="n"/>
+      <c r="J22" s="39" t="n"/>
+      <c r="K22" s="39" t="n"/>
+      <c r="L22" s="39" t="n"/>
+      <c r="M22" s="40" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1" s="1">
-      <c r="A23" s="26" t="n"/>
       <c r="B23" s="22" t="inlineStr">
         <is>
           <t>{belgeTuru} NUMARASI</t>
         </is>
       </c>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="C23" s="40" t="n"/>
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>{belgeNo}</t>
         </is>
       </c>
-      <c r="E23" s="27" t="n"/>
-      <c r="F23" s="27" t="n"/>
-      <c r="G23" s="27" t="n"/>
-      <c r="H23" s="27" t="n"/>
-      <c r="I23" s="27" t="n"/>
-      <c r="J23" s="27" t="n"/>
-      <c r="K23" s="27" t="n"/>
-      <c r="L23" s="27" t="n"/>
-      <c r="M23" s="28" t="n"/>
+      <c r="E23" s="39" t="n"/>
+      <c r="F23" s="39" t="n"/>
+      <c r="G23" s="39" t="n"/>
+      <c r="H23" s="39" t="n"/>
+      <c r="I23" s="39" t="n"/>
+      <c r="J23" s="39" t="n"/>
+      <c r="K23" s="39" t="n"/>
+      <c r="L23" s="39" t="n"/>
+      <c r="M23" s="40" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1" s="1">
-      <c r="A24" s="26" t="n"/>
       <c r="B24" s="22" t="inlineStr">
         <is>
           <t>HAZIRLAYAN</t>
         </is>
       </c>
-      <c r="C24" s="28" t="n"/>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="C24" s="40" t="n"/>
+      <c r="D24" s="42" t="inlineStr">
         <is>
           <t>{hazirlayan}</t>
         </is>
       </c>
-      <c r="E24" s="27" t="n"/>
-      <c r="F24" s="27" t="n"/>
-      <c r="G24" s="27" t="n"/>
-      <c r="H24" s="27" t="n"/>
-      <c r="I24" s="27" t="n"/>
-      <c r="J24" s="27" t="n"/>
-      <c r="K24" s="27" t="n"/>
-      <c r="L24" s="27" t="n"/>
-      <c r="M24" s="28" t="n"/>
+      <c r="E24" s="39" t="n"/>
+      <c r="F24" s="39" t="n"/>
+      <c r="G24" s="39" t="n"/>
+      <c r="H24" s="39" t="n"/>
+      <c r="I24" s="39" t="n"/>
+      <c r="J24" s="39" t="n"/>
+      <c r="K24" s="39" t="n"/>
+      <c r="L24" s="39" t="n"/>
+      <c r="M24" s="40" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1" s="1">
-      <c r="A25" s="26" t="n"/>
       <c r="B25" s="22" t="inlineStr">
         <is>
           <t>GEÇERLİLİK TARİHİ</t>
         </is>
       </c>
-      <c r="C25" s="28" t="n"/>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="42" t="inlineStr">
         <is>
           <t>{gecerlilikTarihi}</t>
         </is>
       </c>
-      <c r="E25" s="27" t="n"/>
-      <c r="F25" s="27" t="n"/>
-      <c r="G25" s="27" t="n"/>
-      <c r="H25" s="27" t="n"/>
-      <c r="I25" s="27" t="n"/>
-      <c r="J25" s="27" t="n"/>
-      <c r="K25" s="27" t="n"/>
-      <c r="L25" s="27" t="n"/>
-      <c r="M25" s="28" t="n"/>
+      <c r="E25" s="39" t="n"/>
+      <c r="F25" s="39" t="n"/>
+      <c r="G25" s="39" t="n"/>
+      <c r="H25" s="39" t="n"/>
+      <c r="I25" s="39" t="n"/>
+      <c r="J25" s="39" t="n"/>
+      <c r="K25" s="39" t="n"/>
+      <c r="L25" s="39" t="n"/>
+      <c r="M25" s="40" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1" s="1">
-      <c r="A26" s="26" t="n"/>
       <c r="B26" s="22" t="inlineStr">
         <is>
           <t>FİYAT LİSTESİ</t>
         </is>
       </c>
-      <c r="C26" s="28" t="n"/>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="C26" s="40" t="n"/>
+      <c r="D26" s="42" t="inlineStr">
         <is>
           <t>{fiyatListesiEtiketi} - Para Birimi: {paraBirimi}</t>
         </is>
       </c>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="27" t="n"/>
-      <c r="G26" s="27" t="n"/>
-      <c r="H26" s="27" t="n"/>
-      <c r="I26" s="27" t="n"/>
-      <c r="J26" s="27" t="n"/>
-      <c r="K26" s="27" t="n"/>
-      <c r="L26" s="27" t="n"/>
-      <c r="M26" s="28" t="n"/>
+      <c r="E26" s="39" t="n"/>
+      <c r="F26" s="39" t="n"/>
+      <c r="G26" s="39" t="n"/>
+      <c r="H26" s="39" t="n"/>
+      <c r="I26" s="39" t="n"/>
+      <c r="J26" s="39" t="n"/>
+      <c r="K26" s="39" t="n"/>
+      <c r="L26" s="39" t="n"/>
+      <c r="M26" s="40" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1" s="1">
       <c r="A27" s="26" t="n"/>
@@ -1370,28 +1375,28 @@
       <c r="L27" s="9" t="n"/>
       <c r="M27" s="9" t="n"/>
     </row>
-    <row r="28" ht="20" customHeight="1" s="1">
+    <row r="28" ht="24" customHeight="1" s="1">
       <c r="A28" s="26" t="n"/>
       <c r="B28" s="15" t="inlineStr">
         <is>
           <t>ÜRÜN GRUPLARI</t>
         </is>
       </c>
-      <c r="C28" s="27" t="n"/>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="27" t="n"/>
-      <c r="G28" s="27" t="n"/>
-      <c r="H28" s="27" t="n"/>
-      <c r="I28" s="27" t="n"/>
-      <c r="J28" s="27" t="n"/>
-      <c r="K28" s="27" t="n"/>
-      <c r="L28" s="27" t="n"/>
-      <c r="M28" s="28" t="n"/>
+      <c r="C28" s="39" t="n"/>
+      <c r="D28" s="39" t="n"/>
+      <c r="E28" s="39" t="n"/>
+      <c r="F28" s="39" t="n"/>
+      <c r="G28" s="39" t="n"/>
+      <c r="H28" s="39" t="n"/>
+      <c r="I28" s="39" t="n"/>
+      <c r="J28" s="39" t="n"/>
+      <c r="K28" s="39" t="n"/>
+      <c r="L28" s="39" t="n"/>
+      <c r="M28" s="40" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1" s="1">
       <c r="A29" s="26" t="n"/>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="43" t="inlineStr">
         <is>
           <t>{urunGruplari}</t>
         </is>
@@ -1438,15 +1443,15 @@
       <c r="L31" s="9" t="n"/>
       <c r="M31" s="9" t="n"/>
     </row>
-    <row r="32" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="32" ht="24" customHeight="1" s="1" thickBot="1">
       <c r="A32" s="26" t="n"/>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="44" t="inlineStr">
         <is>
           <t>YEKÜN İCMAALLERİ</t>
         </is>
       </c>
-      <c r="C32" s="27" t="n"/>
-      <c r="D32" s="28" t="n"/>
+      <c r="C32" s="39" t="n"/>
+      <c r="D32" s="40" t="n"/>
       <c r="E32" s="9" t="n"/>
       <c r="F32" s="9" t="n"/>
       <c r="G32" s="9" t="n"/>
@@ -1457,14 +1462,14 @@
       <c r="L32" s="9" t="n"/>
       <c r="M32" s="9" t="n"/>
     </row>
-    <row r="33" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="33" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A33" s="26" t="n"/>
       <c r="B33" s="22" t="inlineStr">
         <is>
           <t>ÇELİK KAPI GRUBU</t>
         </is>
       </c>
-      <c r="C33" s="28" t="n"/>
+      <c r="C33" s="40" t="n"/>
       <c r="D33" s="30" t="n">
         <v>0</v>
       </c>
@@ -1478,14 +1483,14 @@
       <c r="L33" s="9" t="n"/>
       <c r="M33" s="9" t="n"/>
     </row>
-    <row r="34" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="34" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A34" s="26" t="n"/>
       <c r="B34" s="22" t="inlineStr">
         <is>
           <t>İÇ ODA KAPI GRUBU</t>
         </is>
       </c>
-      <c r="C34" s="28" t="n"/>
+      <c r="C34" s="40" t="n"/>
       <c r="D34" s="30" t="n">
         <v>0</v>
       </c>
@@ -1499,14 +1504,14 @@
       <c r="L34" s="9" t="n"/>
       <c r="M34" s="9" t="n"/>
     </row>
-    <row r="35" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="35" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A35" s="26" t="n"/>
       <c r="B35" s="22" t="inlineStr">
         <is>
           <t>MUTFAK GRUBU</t>
         </is>
       </c>
-      <c r="C35" s="28" t="n"/>
+      <c r="C35" s="40" t="n"/>
       <c r="D35" s="30" t="n">
         <v>0</v>
       </c>
@@ -1520,14 +1525,14 @@
       <c r="L35" s="9" t="n"/>
       <c r="M35" s="9" t="n"/>
     </row>
-    <row r="36" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="36" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A36" s="26" t="n"/>
       <c r="B36" s="22" t="inlineStr">
         <is>
           <t>PORTMANTO GRUBU</t>
         </is>
       </c>
-      <c r="C36" s="28" t="n"/>
+      <c r="C36" s="40" t="n"/>
       <c r="D36" s="30" t="n">
         <v>0</v>
       </c>
@@ -1548,7 +1553,7 @@
           <t>BANYO DOLAPLARI</t>
         </is>
       </c>
-      <c r="C37" s="28" t="n"/>
+      <c r="C37" s="40" t="n"/>
       <c r="D37" s="30" t="n">
         <v>0</v>
       </c>
@@ -1562,14 +1567,14 @@
       <c r="L37" s="9" t="n"/>
       <c r="M37" s="9" t="n"/>
     </row>
-    <row r="38" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="38" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A38" s="26" t="n"/>
       <c r="B38" s="22" t="inlineStr">
         <is>
           <t>AKSESUARLAR</t>
         </is>
       </c>
-      <c r="C38" s="28" t="n"/>
+      <c r="C38" s="40" t="n"/>
       <c r="D38" s="30" t="n">
         <v>0</v>
       </c>
@@ -1583,14 +1588,14 @@
       <c r="L38" s="9" t="n"/>
       <c r="M38" s="9" t="n"/>
     </row>
-    <row r="39" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="39" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A39" s="26" t="n"/>
       <c r="B39" s="22" t="inlineStr">
         <is>
           <t>PARKE</t>
         </is>
       </c>
-      <c r="C39" s="28" t="n"/>
+      <c r="C39" s="40" t="n"/>
       <c r="D39" s="30" t="n">
         <v>0</v>
       </c>
@@ -1604,14 +1609,14 @@
       <c r="L39" s="9" t="n"/>
       <c r="M39" s="9" t="n"/>
     </row>
-    <row r="40" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="40" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A40" s="26" t="n"/>
       <c r="B40" s="22" t="inlineStr">
         <is>
           <t>HİZMETLER &amp; MONTAJ</t>
         </is>
       </c>
-      <c r="C40" s="28" t="n"/>
+      <c r="C40" s="40" t="n"/>
       <c r="D40" s="30" t="n">
         <v>0</v>
       </c>
@@ -1625,14 +1630,14 @@
       <c r="L40" s="9" t="n"/>
       <c r="M40" s="9" t="n"/>
     </row>
-    <row r="41" ht="20" customHeight="1" s="1" thickBot="1">
+    <row r="41" ht="24" customHeight="1" s="1" thickBot="1">
       <c r="A41" s="26" t="n"/>
       <c r="B41" s="22" t="inlineStr">
         <is>
           <t>TOPLAM YEKÜN</t>
         </is>
       </c>
-      <c r="C41" s="28" t="n"/>
+      <c r="C41" s="40" t="n"/>
       <c r="D41" s="30">
         <f>SUM(D33:D40)</f>
         <v/>
@@ -1699,17 +1704,17 @@
           <t>ÖDEME VE TESLİM</t>
         </is>
       </c>
-      <c r="C45" s="27" t="n"/>
-      <c r="D45" s="27" t="n"/>
-      <c r="E45" s="27" t="n"/>
-      <c r="F45" s="27" t="n"/>
-      <c r="G45" s="27" t="n"/>
-      <c r="H45" s="27" t="n"/>
-      <c r="I45" s="27" t="n"/>
-      <c r="J45" s="27" t="n"/>
-      <c r="K45" s="27" t="n"/>
-      <c r="L45" s="27" t="n"/>
-      <c r="M45" s="28" t="n"/>
+      <c r="C45" s="39" t="n"/>
+      <c r="D45" s="39" t="n"/>
+      <c r="E45" s="39" t="n"/>
+      <c r="F45" s="39" t="n"/>
+      <c r="G45" s="39" t="n"/>
+      <c r="H45" s="39" t="n"/>
+      <c r="I45" s="39" t="n"/>
+      <c r="J45" s="39" t="n"/>
+      <c r="K45" s="39" t="n"/>
+      <c r="L45" s="39" t="n"/>
+      <c r="M45" s="40" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1" s="1">
       <c r="A46" s="26" t="n"/>
@@ -1718,21 +1723,21 @@
           <t>ÖDEME KOŞULU</t>
         </is>
       </c>
-      <c r="C46" s="28" t="n"/>
-      <c r="D46" s="11" t="inlineStr">
+      <c r="C46" s="40" t="n"/>
+      <c r="D46" s="42" t="inlineStr">
         <is>
           <t>{odemeKosulu}</t>
         </is>
       </c>
-      <c r="E46" s="27" t="n"/>
-      <c r="F46" s="27" t="n"/>
-      <c r="G46" s="27" t="n"/>
-      <c r="H46" s="27" t="n"/>
-      <c r="I46" s="27" t="n"/>
-      <c r="J46" s="27" t="n"/>
-      <c r="K46" s="27" t="n"/>
-      <c r="L46" s="27" t="n"/>
-      <c r="M46" s="28" t="n"/>
+      <c r="E46" s="39" t="n"/>
+      <c r="F46" s="39" t="n"/>
+      <c r="G46" s="39" t="n"/>
+      <c r="H46" s="39" t="n"/>
+      <c r="I46" s="39" t="n"/>
+      <c r="J46" s="39" t="n"/>
+      <c r="K46" s="39" t="n"/>
+      <c r="L46" s="39" t="n"/>
+      <c r="M46" s="40" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1" s="1">
       <c r="A47" s="26" t="n"/>
@@ -1741,21 +1746,21 @@
           <t>TESLİM TİPİ</t>
         </is>
       </c>
-      <c r="C47" s="28" t="n"/>
-      <c r="D47" s="11" t="inlineStr">
+      <c r="C47" s="40" t="n"/>
+      <c r="D47" s="42" t="inlineStr">
         <is>
           <t>{teslimTipi}</t>
         </is>
       </c>
-      <c r="E47" s="27" t="n"/>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
-      <c r="I47" s="27" t="n"/>
-      <c r="J47" s="27" t="n"/>
-      <c r="K47" s="27" t="n"/>
-      <c r="L47" s="27" t="n"/>
-      <c r="M47" s="28" t="n"/>
+      <c r="E47" s="39" t="n"/>
+      <c r="F47" s="39" t="n"/>
+      <c r="G47" s="39" t="n"/>
+      <c r="H47" s="39" t="n"/>
+      <c r="I47" s="39" t="n"/>
+      <c r="J47" s="39" t="n"/>
+      <c r="K47" s="39" t="n"/>
+      <c r="L47" s="39" t="n"/>
+      <c r="M47" s="40" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1" s="1">
       <c r="A48" s="26" t="n"/>
@@ -1764,21 +1769,21 @@
           <t>TESLİM TARİHİ</t>
         </is>
       </c>
-      <c r="C48" s="28" t="n"/>
-      <c r="D48" s="11" t="inlineStr">
+      <c r="C48" s="40" t="n"/>
+      <c r="D48" s="42" t="inlineStr">
         <is>
           <t>{teslimTarihi}</t>
         </is>
       </c>
-      <c r="E48" s="27" t="n"/>
-      <c r="F48" s="27" t="n"/>
-      <c r="G48" s="27" t="n"/>
-      <c r="H48" s="27" t="n"/>
-      <c r="I48" s="27" t="n"/>
-      <c r="J48" s="27" t="n"/>
-      <c r="K48" s="27" t="n"/>
-      <c r="L48" s="27" t="n"/>
-      <c r="M48" s="28" t="n"/>
+      <c r="E48" s="39" t="n"/>
+      <c r="F48" s="39" t="n"/>
+      <c r="G48" s="39" t="n"/>
+      <c r="H48" s="39" t="n"/>
+      <c r="I48" s="39" t="n"/>
+      <c r="J48" s="39" t="n"/>
+      <c r="K48" s="39" t="n"/>
+      <c r="L48" s="39" t="n"/>
+      <c r="M48" s="40" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1" s="1">
       <c r="A49" s="26" t="n"/>
@@ -1787,21 +1792,21 @@
           <t>NOTLAR</t>
         </is>
       </c>
-      <c r="C49" s="28" t="n"/>
-      <c r="D49" s="11" t="inlineStr">
+      <c r="C49" s="40" t="n"/>
+      <c r="D49" s="42" t="inlineStr">
         <is>
           <t>{notlar}</t>
         </is>
       </c>
-      <c r="E49" s="27" t="n"/>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="27" t="n"/>
-      <c r="I49" s="27" t="n"/>
-      <c r="J49" s="27" t="n"/>
-      <c r="K49" s="27" t="n"/>
-      <c r="L49" s="27" t="n"/>
-      <c r="M49" s="28" t="n"/>
+      <c r="E49" s="39" t="n"/>
+      <c r="F49" s="39" t="n"/>
+      <c r="G49" s="39" t="n"/>
+      <c r="H49" s="39" t="n"/>
+      <c r="I49" s="39" t="n"/>
+      <c r="J49" s="39" t="n"/>
+      <c r="K49" s="39" t="n"/>
+      <c r="L49" s="39" t="n"/>
+      <c r="M49" s="40" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1" s="1">
       <c r="A50" s="26" t="n"/>
@@ -1840,109 +1845,109 @@
           <t>FİRMA ÜNVANI &amp; IBANLAR</t>
         </is>
       </c>
-      <c r="C52" s="27" t="n"/>
-      <c r="D52" s="27" t="n"/>
-      <c r="E52" s="27" t="n"/>
-      <c r="F52" s="27" t="n"/>
-      <c r="G52" s="27" t="n"/>
-      <c r="H52" s="27" t="n"/>
-      <c r="I52" s="27" t="n"/>
-      <c r="J52" s="27" t="n"/>
-      <c r="K52" s="27" t="n"/>
-      <c r="L52" s="27" t="n"/>
-      <c r="M52" s="28" t="n"/>
+      <c r="C52" s="39" t="n"/>
+      <c r="D52" s="39" t="n"/>
+      <c r="E52" s="39" t="n"/>
+      <c r="F52" s="39" t="n"/>
+      <c r="G52" s="39" t="n"/>
+      <c r="H52" s="39" t="n"/>
+      <c r="I52" s="39" t="n"/>
+      <c r="J52" s="39" t="n"/>
+      <c r="K52" s="39" t="n"/>
+      <c r="L52" s="39" t="n"/>
+      <c r="M52" s="40" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1" s="1">
       <c r="A53" s="26" t="n"/>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B53" s="22" t="inlineStr">
         <is>
           <t>{seciliSatici.banka1.ad}</t>
         </is>
       </c>
-      <c r="C53" s="28" t="n"/>
-      <c r="D53" s="11" t="inlineStr">
+      <c r="C53" s="40" t="n"/>
+      <c r="D53" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.banka1.iban}</t>
         </is>
       </c>
-      <c r="E53" s="27" t="n"/>
-      <c r="F53" s="27" t="n"/>
-      <c r="G53" s="27" t="n"/>
-      <c r="H53" s="27" t="n"/>
-      <c r="I53" s="27" t="n"/>
-      <c r="J53" s="27" t="n"/>
-      <c r="K53" s="27" t="n"/>
-      <c r="L53" s="27" t="n"/>
-      <c r="M53" s="28" t="n"/>
+      <c r="E53" s="39" t="n"/>
+      <c r="F53" s="39" t="n"/>
+      <c r="G53" s="39" t="n"/>
+      <c r="H53" s="39" t="n"/>
+      <c r="I53" s="39" t="n"/>
+      <c r="J53" s="39" t="n"/>
+      <c r="K53" s="39" t="n"/>
+      <c r="L53" s="39" t="n"/>
+      <c r="M53" s="40" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1" s="1">
       <c r="A54" s="26" t="n"/>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>{seciliSatici.banka2.ad}</t>
         </is>
       </c>
-      <c r="C54" s="28" t="n"/>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="C54" s="40" t="n"/>
+      <c r="D54" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.banka2.iban}</t>
         </is>
       </c>
-      <c r="E54" s="27" t="n"/>
-      <c r="F54" s="27" t="n"/>
-      <c r="G54" s="27" t="n"/>
-      <c r="H54" s="27" t="n"/>
-      <c r="I54" s="27" t="n"/>
-      <c r="J54" s="27" t="n"/>
-      <c r="K54" s="27" t="n"/>
-      <c r="L54" s="27" t="n"/>
-      <c r="M54" s="28" t="n"/>
+      <c r="E54" s="39" t="n"/>
+      <c r="F54" s="39" t="n"/>
+      <c r="G54" s="39" t="n"/>
+      <c r="H54" s="39" t="n"/>
+      <c r="I54" s="39" t="n"/>
+      <c r="J54" s="39" t="n"/>
+      <c r="K54" s="39" t="n"/>
+      <c r="L54" s="39" t="n"/>
+      <c r="M54" s="40" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1" s="1">
       <c r="A55" s="26" t="n"/>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>{seciliSatici.banka3.ad}</t>
         </is>
       </c>
-      <c r="C55" s="28" t="n"/>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="C55" s="40" t="n"/>
+      <c r="D55" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.banka3.iban}</t>
         </is>
       </c>
-      <c r="E55" s="27" t="n"/>
-      <c r="F55" s="27" t="n"/>
-      <c r="G55" s="27" t="n"/>
-      <c r="H55" s="27" t="n"/>
-      <c r="I55" s="27" t="n"/>
-      <c r="J55" s="27" t="n"/>
-      <c r="K55" s="27" t="n"/>
-      <c r="L55" s="27" t="n"/>
-      <c r="M55" s="28" t="n"/>
+      <c r="E55" s="39" t="n"/>
+      <c r="F55" s="39" t="n"/>
+      <c r="G55" s="39" t="n"/>
+      <c r="H55" s="39" t="n"/>
+      <c r="I55" s="39" t="n"/>
+      <c r="J55" s="39" t="n"/>
+      <c r="K55" s="39" t="n"/>
+      <c r="L55" s="39" t="n"/>
+      <c r="M55" s="40" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1" s="1">
       <c r="A56" s="26" t="n"/>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="B56" s="22" t="inlineStr">
         <is>
           <t>{seciliSatici.banka4.ad}</t>
         </is>
       </c>
-      <c r="C56" s="28" t="n"/>
-      <c r="D56" s="11" t="inlineStr">
+      <c r="C56" s="40" t="n"/>
+      <c r="D56" s="42" t="inlineStr">
         <is>
           <t>{seciliSatici.banka4.iban}</t>
         </is>
       </c>
-      <c r="E56" s="27" t="n"/>
-      <c r="F56" s="27" t="n"/>
-      <c r="G56" s="27" t="n"/>
-      <c r="H56" s="27" t="n"/>
-      <c r="I56" s="27" t="n"/>
-      <c r="J56" s="27" t="n"/>
-      <c r="K56" s="27" t="n"/>
-      <c r="L56" s="27" t="n"/>
-      <c r="M56" s="28" t="n"/>
+      <c r="E56" s="39" t="n"/>
+      <c r="F56" s="39" t="n"/>
+      <c r="G56" s="39" t="n"/>
+      <c r="H56" s="39" t="n"/>
+      <c r="I56" s="39" t="n"/>
+      <c r="J56" s="39" t="n"/>
+      <c r="K56" s="39" t="n"/>
+      <c r="L56" s="39" t="n"/>
+      <c r="M56" s="40" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1" s="1">
       <c r="A57" s="26" t="n"/>
@@ -1996,117 +2001,85 @@
           <t>TARAFLARIN KAŞE İMZASI</t>
         </is>
       </c>
-      <c r="C60" s="27" t="n"/>
-      <c r="D60" s="27" t="n"/>
-      <c r="E60" s="27" t="n"/>
-      <c r="F60" s="27" t="n"/>
-      <c r="G60" s="27" t="n"/>
-      <c r="H60" s="27" t="n"/>
-      <c r="I60" s="27" t="n"/>
-      <c r="J60" s="27" t="n"/>
-      <c r="K60" s="27" t="n"/>
-      <c r="L60" s="27" t="n"/>
-      <c r="M60" s="28" t="n"/>
+      <c r="C60" s="39" t="n"/>
+      <c r="D60" s="39" t="n"/>
+      <c r="E60" s="39" t="n"/>
+      <c r="F60" s="39" t="n"/>
+      <c r="G60" s="39" t="n"/>
+      <c r="H60" s="39" t="n"/>
+      <c r="I60" s="39" t="n"/>
+      <c r="J60" s="39" t="n"/>
+      <c r="K60" s="39" t="n"/>
+      <c r="L60" s="39" t="n"/>
+      <c r="M60" s="40" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1" s="1">
       <c r="A61" s="26" t="n"/>
-      <c r="B61" s="24" t="inlineStr">
+      <c r="B61" s="45" t="inlineStr">
         <is>
           <t>SATICI
 {seciliSatici.resmiUnvan}</t>
         </is>
       </c>
-      <c r="C61" s="31" t="n"/>
-      <c r="D61" s="31" t="n"/>
-      <c r="E61" s="31" t="n"/>
-      <c r="F61" s="31" t="n"/>
-      <c r="G61" s="32" t="n"/>
-      <c r="H61" s="24" t="inlineStr">
+      <c r="C61" s="46" t="n"/>
+      <c r="D61" s="46" t="n"/>
+      <c r="E61" s="46" t="n"/>
+      <c r="F61" s="46" t="n"/>
+      <c r="G61" s="47" t="n"/>
+      <c r="H61" s="45" t="inlineStr">
         <is>
           <t>ALICI
 {cariUnvani}</t>
         </is>
       </c>
-      <c r="I61" s="31" t="n"/>
-      <c r="J61" s="31" t="n"/>
-      <c r="K61" s="31" t="n"/>
-      <c r="L61" s="31" t="n"/>
-      <c r="M61" s="32" t="n"/>
+      <c r="I61" s="46" t="n"/>
+      <c r="J61" s="46" t="n"/>
+      <c r="K61" s="46" t="n"/>
+      <c r="L61" s="46" t="n"/>
+      <c r="M61" s="47" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1" s="1">
       <c r="A62" s="26" t="n"/>
-      <c r="B62" s="33" t="n"/>
-      <c r="C62" s="26" t="n"/>
-      <c r="D62" s="26" t="n"/>
-      <c r="E62" s="26" t="n"/>
-      <c r="F62" s="26" t="n"/>
-      <c r="G62" s="34" t="n"/>
-      <c r="H62" s="33" t="n"/>
-      <c r="I62" s="26" t="n"/>
-      <c r="J62" s="26" t="n"/>
-      <c r="K62" s="26" t="n"/>
-      <c r="L62" s="26" t="n"/>
-      <c r="M62" s="34" t="n"/>
+      <c r="B62" s="48" t="n"/>
+      <c r="G62" s="49" t="n"/>
+      <c r="H62" s="48" t="n"/>
+      <c r="M62" s="49" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1" s="1">
       <c r="A63" s="26" t="n"/>
-      <c r="B63" s="33" t="n"/>
-      <c r="C63" s="26" t="n"/>
-      <c r="D63" s="26" t="n"/>
-      <c r="E63" s="26" t="n"/>
-      <c r="F63" s="26" t="n"/>
-      <c r="G63" s="34" t="n"/>
-      <c r="H63" s="33" t="n"/>
-      <c r="I63" s="26" t="n"/>
-      <c r="J63" s="26" t="n"/>
-      <c r="K63" s="26" t="n"/>
-      <c r="L63" s="26" t="n"/>
-      <c r="M63" s="34" t="n"/>
+      <c r="B63" s="48" t="n"/>
+      <c r="G63" s="49" t="n"/>
+      <c r="H63" s="48" t="n"/>
+      <c r="M63" s="49" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1" s="1">
       <c r="A64" s="26" t="n"/>
-      <c r="B64" s="33" t="n"/>
-      <c r="C64" s="26" t="n"/>
-      <c r="D64" s="26" t="n"/>
-      <c r="E64" s="26" t="n"/>
-      <c r="F64" s="26" t="n"/>
-      <c r="G64" s="34" t="n"/>
-      <c r="H64" s="33" t="n"/>
-      <c r="I64" s="26" t="n"/>
-      <c r="J64" s="26" t="n"/>
-      <c r="K64" s="26" t="n"/>
-      <c r="L64" s="26" t="n"/>
-      <c r="M64" s="34" t="n"/>
+      <c r="B64" s="48" t="n"/>
+      <c r="G64" s="49" t="n"/>
+      <c r="H64" s="48" t="n"/>
+      <c r="M64" s="49" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1" s="1">
       <c r="A65" s="26" t="n"/>
-      <c r="B65" s="33" t="n"/>
-      <c r="C65" s="26" t="n"/>
-      <c r="D65" s="26" t="n"/>
-      <c r="E65" s="26" t="n"/>
-      <c r="F65" s="26" t="n"/>
-      <c r="G65" s="34" t="n"/>
-      <c r="H65" s="33" t="n"/>
-      <c r="I65" s="26" t="n"/>
-      <c r="J65" s="26" t="n"/>
-      <c r="K65" s="26" t="n"/>
-      <c r="L65" s="26" t="n"/>
-      <c r="M65" s="34" t="n"/>
+      <c r="B65" s="48" t="n"/>
+      <c r="G65" s="49" t="n"/>
+      <c r="H65" s="48" t="n"/>
+      <c r="M65" s="49" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1" s="1">
       <c r="A66" s="26" t="n"/>
-      <c r="B66" s="35" t="n"/>
-      <c r="C66" s="36" t="n"/>
-      <c r="D66" s="36" t="n"/>
-      <c r="E66" s="36" t="n"/>
-      <c r="F66" s="36" t="n"/>
-      <c r="G66" s="37" t="n"/>
-      <c r="H66" s="35" t="n"/>
-      <c r="I66" s="36" t="n"/>
-      <c r="J66" s="36" t="n"/>
-      <c r="K66" s="36" t="n"/>
-      <c r="L66" s="36" t="n"/>
-      <c r="M66" s="37" t="n"/>
+      <c r="B66" s="50" t="n"/>
+      <c r="C66" s="51" t="n"/>
+      <c r="D66" s="51" t="n"/>
+      <c r="E66" s="51" t="n"/>
+      <c r="F66" s="51" t="n"/>
+      <c r="G66" s="52" t="n"/>
+      <c r="H66" s="50" t="n"/>
+      <c r="I66" s="51" t="n"/>
+      <c r="J66" s="51" t="n"/>
+      <c r="K66" s="51" t="n"/>
+      <c r="L66" s="51" t="n"/>
+      <c r="M66" s="52" t="n"/>
     </row>
     <row r="67" ht="20" customHeight="1" s="1">
       <c r="A67" s="26" t="n"/>
@@ -2154,9 +2127,9 @@
     <mergeCell ref="D25:M25"/>
     <mergeCell ref="B2:E5"/>
     <mergeCell ref="B56:C56"/>
+    <mergeCell ref="D55:M55"/>
+    <mergeCell ref="D24:M24"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D24:M24"/>
-    <mergeCell ref="D55:M55"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="D23:M23"/>

</xml_diff>

<commit_message>
update seller buyer contract layout
</commit_message>
<xml_diff>
--- a/backend/crm/assets/contract-templates/MASTER/SELLER_MASTER_TEMPLATE.xlsx
+++ b/backend/crm/assets/contract-templates/MASTER/SELLER_MASTER_TEMPLATE.xlsx
@@ -1,14 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="19180" windowHeight="7160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Belge" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Belge" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Belge'!$B$1:$M$55</definedName>
+  </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;₺&quot;* #,##0.00_-;\-&quot;₺&quot;* #,##0.00_-;_-&quot;₺&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -174,6 +176,14 @@
       <b val="1"/>
       <color rgb="FF203864"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <charset val="162"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -194,7 +204,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -323,12 +333,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -434,6 +455,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +537,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>0</col>
@@ -530,25 +555,25 @@
       <nvPicPr>
         <cNvPr id="2" name="Resim 1"/>
         <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill rotWithShape="1">
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" t="71298"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:srcRect t="71298"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:xfrm>
           <a:off x="234951" y="19577692"/>
           <a:ext cx="12560300" cy="1006287"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+        <a:prstGeom prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -847,17 +872,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="4" customWidth="1" style="1" min="1" max="1"/>
-    <col width="15" customWidth="1" style="1" min="2" max="3"/>
-    <col width="20" customWidth="1" style="1" min="4" max="4"/>
-    <col width="15" customWidth="1" style="1" min="5" max="6"/>
-    <col width="12" customWidth="1" style="1" min="7" max="9"/>
-    <col width="14" customWidth="1" style="1" min="10" max="10"/>
-    <col width="15" customWidth="1" style="1" min="11" max="11"/>
-    <col width="18" customWidth="1" style="1" min="12" max="13"/>
+    <col hidden="1" width="4" customWidth="1" style="1" min="1" max="1"/>
+    <col width="13" customWidth="1" style="1" min="2" max="3"/>
+    <col width="14" customWidth="1" style="1" min="3" max="3"/>
+    <col width="17" customWidth="1" style="1" min="4" max="4"/>
+    <col width="13" customWidth="1" style="1" min="5" max="6"/>
+    <col width="13" customWidth="1" style="1" min="6" max="6"/>
+    <col width="11" customWidth="1" style="1" min="7" max="9"/>
+    <col width="11" customWidth="1" style="1" min="8" max="8"/>
+    <col width="11" customWidth="1" style="1" min="9" max="9"/>
+    <col width="13" customWidth="1" style="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="1" min="11" max="11"/>
+    <col width="15" customWidth="1" style="1" min="12" max="13"/>
+    <col width="16" customWidth="1" style="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" s="1">
@@ -886,11 +916,14 @@
       <c r="G2" s="26" t="n"/>
       <c r="H2" s="26" t="n"/>
       <c r="I2" s="26" t="n"/>
-      <c r="J2" s="38" t="inlineStr">
-        <is>
-          <t>{seciliSatici.resmiUnvan}</t>
-        </is>
-      </c>
+      <c r="J2" s="53" t="inlineStr">
+        <is>
+          <t>DETAYLAR</t>
+        </is>
+      </c>
+      <c r="K2" s="39" t="n"/>
+      <c r="L2" s="39" t="n"/>
+      <c r="M2" s="40" t="n"/>
     </row>
     <row r="3" ht="23" customHeight="1" s="1">
       <c r="A3" s="26" t="n"/>
@@ -898,6 +931,18 @@
       <c r="G3" s="26" t="n"/>
       <c r="H3" s="26" t="n"/>
       <c r="I3" s="26" t="n"/>
+      <c r="J3" s="22" t="inlineStr">
+        <is>
+          <t>{belgeTuru} NO</t>
+        </is>
+      </c>
+      <c r="K3" s="40" t="n"/>
+      <c r="L3" s="42" t="inlineStr">
+        <is>
+          <t>{belgeNo}</t>
+        </is>
+      </c>
+      <c r="M3" s="40" t="n"/>
     </row>
     <row r="4" ht="23" customHeight="1" s="1">
       <c r="A4" s="26" t="n"/>
@@ -905,11 +950,18 @@
       <c r="G4" s="26" t="n"/>
       <c r="H4" s="26" t="n"/>
       <c r="I4" s="26" t="n"/>
-      <c r="J4" s="38" t="inlineStr">
-        <is>
-          <t>{seciliSatici.kisaAd}</t>
-        </is>
-      </c>
+      <c r="J4" s="22" t="inlineStr">
+        <is>
+          <t>TARİH</t>
+        </is>
+      </c>
+      <c r="K4" s="40" t="n"/>
+      <c r="L4" s="42" t="inlineStr">
+        <is>
+          <t>{olusturmaTarihi}</t>
+        </is>
+      </c>
+      <c r="M4" s="40" t="n"/>
     </row>
     <row r="5" ht="23" customHeight="1" s="1">
       <c r="A5" s="26" t="n"/>
@@ -917,11 +969,18 @@
       <c r="G5" s="26" t="n"/>
       <c r="H5" s="26" t="n"/>
       <c r="I5" s="26" t="n"/>
-      <c r="J5" s="38" t="inlineStr">
-        <is>
-          <t>{seciliSatici.email} / {seciliSatici.telefon}</t>
-        </is>
-      </c>
+      <c r="J5" s="22" t="inlineStr">
+        <is>
+          <t>HAZIRLAYAN</t>
+        </is>
+      </c>
+      <c r="K5" s="40" t="n"/>
+      <c r="L5" s="42" t="inlineStr">
+        <is>
+          <t>{hazirlayan}</t>
+        </is>
+      </c>
+      <c r="M5" s="40" t="n"/>
     </row>
     <row r="6" ht="23" customHeight="1" s="1">
       <c r="A6" s="26" t="n"/>
@@ -958,59 +1017,43 @@
       <c r="M7" s="40" t="n"/>
     </row>
     <row r="8" ht="23" customHeight="1" s="1">
-      <c r="A8" s="26" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="41" t="inlineStr">
-        <is>
-          <t>TARİH</t>
-        </is>
-      </c>
-      <c r="L8" s="40" t="n"/>
-      <c r="M8" s="41" t="inlineStr">
-        <is>
-          <t>{olusturmaTarihi}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1" s="1">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>T
-A
-R
-A
-F
-L
-A
-R</t>
-        </is>
-      </c>
+      <c r="A8" s="26" t="inlineStr"/>
+      <c r="B8" s="9" t="inlineStr"/>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr"/>
+      <c r="K8" s="41" t="inlineStr"/>
+      <c r="M8" s="41" t="inlineStr"/>
+    </row>
+    <row r="9" ht="28" customHeight="1" s="1">
+      <c r="A9" s="29" t="inlineStr"/>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>SATIŞI YAPAN FİRMA</t>
+          <t>SATICI BİLGİLERİ</t>
         </is>
       </c>
       <c r="C9" s="39" t="n"/>
       <c r="D9" s="39" t="n"/>
       <c r="E9" s="39" t="n"/>
       <c r="F9" s="39" t="n"/>
-      <c r="G9" s="39" t="n"/>
-      <c r="H9" s="39" t="n"/>
+      <c r="G9" s="40" t="n"/>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>ALICI BİLGİLERİ</t>
+        </is>
+      </c>
       <c r="I9" s="39" t="n"/>
       <c r="J9" s="39" t="n"/>
       <c r="K9" s="39" t="n"/>
       <c r="L9" s="39" t="n"/>
       <c r="M9" s="40" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1" s="1">
+    <row r="10" ht="28" customHeight="1" s="1">
       <c r="B10" s="22" t="inlineStr">
         <is>
           <t>ÜNVAN</t>
@@ -1024,15 +1067,23 @@
       </c>
       <c r="E10" s="39" t="n"/>
       <c r="F10" s="39" t="n"/>
-      <c r="G10" s="39" t="n"/>
-      <c r="H10" s="39" t="n"/>
-      <c r="I10" s="39" t="n"/>
-      <c r="J10" s="39" t="n"/>
+      <c r="G10" s="40" t="n"/>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>CARİ ÜNVANI</t>
+        </is>
+      </c>
+      <c r="I10" s="40" t="n"/>
+      <c r="J10" s="42" t="inlineStr">
+        <is>
+          <t>{cariUnvani}</t>
+        </is>
+      </c>
       <c r="K10" s="39" t="n"/>
       <c r="L10" s="39" t="n"/>
       <c r="M10" s="40" t="n"/>
     </row>
-    <row r="11" ht="24" customHeight="1" s="1">
+    <row r="11" ht="28" customHeight="1" s="1">
       <c r="B11" s="22" t="inlineStr">
         <is>
           <t>VERGİ DAİRESİ / NO</t>
@@ -1046,15 +1097,23 @@
       </c>
       <c r="E11" s="39" t="n"/>
       <c r="F11" s="39" t="n"/>
-      <c r="G11" s="39" t="n"/>
-      <c r="H11" s="39" t="n"/>
-      <c r="I11" s="39" t="n"/>
-      <c r="J11" s="39" t="n"/>
+      <c r="G11" s="40" t="n"/>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t>VERGİ DAİRESİ / NO</t>
+        </is>
+      </c>
+      <c r="I11" s="40" t="n"/>
+      <c r="J11" s="42" t="inlineStr">
+        <is>
+          <t>{vergiDairesi} / {vergiNo}</t>
+        </is>
+      </c>
       <c r="K11" s="39" t="n"/>
       <c r="L11" s="39" t="n"/>
       <c r="M11" s="40" t="n"/>
     </row>
-    <row r="12" ht="20" customHeight="1" s="1">
+    <row r="12" ht="28" customHeight="1" s="1">
       <c r="B12" s="22" t="inlineStr">
         <is>
           <t>ADRES</t>
@@ -1068,15 +1127,23 @@
       </c>
       <c r="E12" s="39" t="n"/>
       <c r="F12" s="39" t="n"/>
-      <c r="G12" s="39" t="n"/>
-      <c r="H12" s="39" t="n"/>
-      <c r="I12" s="39" t="n"/>
-      <c r="J12" s="39" t="n"/>
+      <c r="G12" s="40" t="n"/>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>ADRES</t>
+        </is>
+      </c>
+      <c r="I12" s="40" t="n"/>
+      <c r="J12" s="42" t="inlineStr">
+        <is>
+          <t>{adres}</t>
+        </is>
+      </c>
       <c r="K12" s="39" t="n"/>
       <c r="L12" s="39" t="n"/>
       <c r="M12" s="40" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1" s="1">
+    <row r="13" ht="28" customHeight="1" s="1">
       <c r="B13" s="22" t="inlineStr">
         <is>
           <t>TELEFON / E-POSTA</t>
@@ -1090,32 +1157,49 @@
       </c>
       <c r="E13" s="39" t="n"/>
       <c r="F13" s="39" t="n"/>
-      <c r="G13" s="39" t="n"/>
-      <c r="H13" s="39" t="n"/>
-      <c r="I13" s="39" t="n"/>
-      <c r="J13" s="39" t="n"/>
+      <c r="G13" s="40" t="n"/>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>YETKİLİ</t>
+        </is>
+      </c>
+      <c r="I13" s="40" t="n"/>
+      <c r="J13" s="42" t="inlineStr">
+        <is>
+          <t>{yetkili}</t>
+        </is>
+      </c>
       <c r="K13" s="39" t="n"/>
       <c r="L13" s="39" t="n"/>
       <c r="M13" s="40" t="n"/>
     </row>
-    <row r="14" ht="20" customHeight="1" s="1">
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
-      <c r="M14" s="9" t="n"/>
+    <row r="14" ht="28" customHeight="1" s="1">
+      <c r="B14" s="22" t="inlineStr"/>
+      <c r="C14" s="40" t="n"/>
+      <c r="D14" s="42" t="inlineStr"/>
+      <c r="E14" s="39" t="n"/>
+      <c r="F14" s="39" t="n"/>
+      <c r="G14" s="40" t="n"/>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>TELEFON / E-POSTA</t>
+        </is>
+      </c>
+      <c r="I14" s="40" t="n"/>
+      <c r="J14" s="42" t="inlineStr">
+        <is>
+          <t>{telefon} / {email}</t>
+        </is>
+      </c>
+      <c r="K14" s="39" t="n"/>
+      <c r="L14" s="39" t="n"/>
+      <c r="M14" s="40" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1" s="1">
+      <c r="A15" s="26" t="n"/>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>ALICI BİLGİLERİ</t>
+          <t>ÜRÜN GRUPLARI</t>
         </is>
       </c>
       <c r="C15" s="39" t="n"/>
@@ -1131,119 +1215,105 @@
       <c r="M15" s="40" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1" s="1">
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>CARİ ÜNVANI</t>
-        </is>
-      </c>
-      <c r="C16" s="40" t="n"/>
-      <c r="D16" s="42" t="inlineStr">
-        <is>
-          <t>{cariUnvani}</t>
-        </is>
-      </c>
-      <c r="E16" s="39" t="n"/>
-      <c r="F16" s="39" t="n"/>
-      <c r="G16" s="39" t="n"/>
-      <c r="H16" s="39" t="n"/>
-      <c r="I16" s="39" t="n"/>
-      <c r="J16" s="39" t="n"/>
-      <c r="K16" s="39" t="n"/>
-      <c r="L16" s="39" t="n"/>
-      <c r="M16" s="40" t="n"/>
+      <c r="A16" s="26" t="n"/>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>{urunGruplari}</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="9" t="n"/>
+      <c r="M16" s="9" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1" s="1">
-      <c r="B17" s="22" t="inlineStr">
-        <is>
-          <t>VERGİ DAİRESİ / NO</t>
-        </is>
-      </c>
-      <c r="C17" s="40" t="n"/>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>{vergiDairesi} / {vergiNo}</t>
-        </is>
-      </c>
-      <c r="E17" s="39" t="n"/>
-      <c r="F17" s="39" t="n"/>
-      <c r="G17" s="39" t="n"/>
-      <c r="H17" s="39" t="n"/>
-      <c r="I17" s="39" t="n"/>
-      <c r="J17" s="39" t="n"/>
-      <c r="K17" s="39" t="n"/>
-      <c r="L17" s="39" t="n"/>
-      <c r="M17" s="40" t="n"/>
+      <c r="A17" s="26" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="9" t="n"/>
+      <c r="M17" s="9" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1" s="1">
-      <c r="B18" s="22" t="inlineStr">
-        <is>
-          <t>ADRES</t>
-        </is>
-      </c>
-      <c r="C18" s="40" t="n"/>
-      <c r="D18" s="42" t="inlineStr">
-        <is>
-          <t>{adres}</t>
-        </is>
-      </c>
-      <c r="E18" s="39" t="n"/>
-      <c r="F18" s="39" t="n"/>
-      <c r="G18" s="39" t="n"/>
-      <c r="H18" s="39" t="n"/>
-      <c r="I18" s="39" t="n"/>
-      <c r="J18" s="39" t="n"/>
-      <c r="K18" s="39" t="n"/>
-      <c r="L18" s="39" t="n"/>
-      <c r="M18" s="40" t="n"/>
+      <c r="A18" s="26" t="n"/>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="9" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="9" t="n"/>
+      <c r="L18" s="9" t="n"/>
+      <c r="M18" s="9" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1" s="1">
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>YETKİLİ</t>
-        </is>
-      </c>
-      <c r="C19" s="40" t="n"/>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>{yetkili}</t>
-        </is>
-      </c>
-      <c r="E19" s="39" t="n"/>
-      <c r="F19" s="39" t="n"/>
-      <c r="G19" s="39" t="n"/>
-      <c r="H19" s="39" t="n"/>
-      <c r="I19" s="39" t="n"/>
-      <c r="J19" s="39" t="n"/>
-      <c r="K19" s="39" t="n"/>
-      <c r="L19" s="39" t="n"/>
-      <c r="M19" s="40" t="n"/>
+      <c r="A19" s="26" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>YEKÜN İCMAALLERİ</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="40" t="n"/>
+      <c r="E19" s="9" t="n"/>
+      <c r="F19" s="9" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="9" t="n"/>
+      <c r="L19" s="9" t="n"/>
+      <c r="M19" s="9" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1" s="1">
+      <c r="A20" s="26" t="n"/>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>TELEFON / E-POSTA</t>
+          <t>ÇELİK KAPI GRUBU</t>
         </is>
       </c>
       <c r="C20" s="40" t="n"/>
-      <c r="D20" s="42" t="inlineStr">
-        <is>
-          <t>{telefon} / {email}</t>
-        </is>
-      </c>
-      <c r="E20" s="39" t="n"/>
-      <c r="F20" s="39" t="n"/>
-      <c r="G20" s="39" t="n"/>
-      <c r="H20" s="39" t="n"/>
-      <c r="I20" s="39" t="n"/>
-      <c r="J20" s="39" t="n"/>
-      <c r="K20" s="39" t="n"/>
-      <c r="L20" s="39" t="n"/>
-      <c r="M20" s="40" t="n"/>
+      <c r="D20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="9" t="n"/>
+      <c r="F20" s="9" t="n"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" s="9" t="n"/>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="9" t="n"/>
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="9" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1" s="1">
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
+      <c r="A21" s="26" t="n"/>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>İÇ ODA KAPI GRUBU</t>
+        </is>
+      </c>
+      <c r="C21" s="40" t="n"/>
+      <c r="D21" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" s="9" t="n"/>
       <c r="F21" s="9" t="n"/>
       <c r="G21" s="9" t="n"/>
@@ -1255,116 +1325,121 @@
       <c r="M21" s="9" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1" s="1">
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>{belgeTuru} DETAYLARI</t>
-        </is>
-      </c>
-      <c r="C22" s="39" t="n"/>
-      <c r="D22" s="39" t="n"/>
-      <c r="E22" s="39" t="n"/>
-      <c r="F22" s="39" t="n"/>
-      <c r="G22" s="39" t="n"/>
-      <c r="H22" s="39" t="n"/>
-      <c r="I22" s="39" t="n"/>
-      <c r="J22" s="39" t="n"/>
-      <c r="K22" s="39" t="n"/>
-      <c r="L22" s="39" t="n"/>
-      <c r="M22" s="40" t="n"/>
+      <c r="A22" s="26" t="n"/>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>MUTFAK GRUBU</t>
+        </is>
+      </c>
+      <c r="C22" s="40" t="n"/>
+      <c r="D22" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1" s="1">
+      <c r="A23" s="26" t="n"/>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>{belgeTuru} NUMARASI</t>
+          <t>PORTMANTO GRUBU</t>
         </is>
       </c>
       <c r="C23" s="40" t="n"/>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>{belgeNo}</t>
-        </is>
-      </c>
-      <c r="E23" s="39" t="n"/>
-      <c r="F23" s="39" t="n"/>
-      <c r="G23" s="39" t="n"/>
-      <c r="H23" s="39" t="n"/>
-      <c r="I23" s="39" t="n"/>
-      <c r="J23" s="39" t="n"/>
-      <c r="K23" s="39" t="n"/>
-      <c r="L23" s="39" t="n"/>
-      <c r="M23" s="40" t="n"/>
+      <c r="D23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1" s="1">
+      <c r="A24" s="26" t="n"/>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>HAZIRLAYAN</t>
+          <t>BANYO DOLAPLARI</t>
         </is>
       </c>
       <c r="C24" s="40" t="n"/>
-      <c r="D24" s="42" t="inlineStr">
-        <is>
-          <t>{hazirlayan}</t>
-        </is>
-      </c>
-      <c r="E24" s="39" t="n"/>
-      <c r="F24" s="39" t="n"/>
-      <c r="G24" s="39" t="n"/>
-      <c r="H24" s="39" t="n"/>
-      <c r="I24" s="39" t="n"/>
-      <c r="J24" s="39" t="n"/>
-      <c r="K24" s="39" t="n"/>
-      <c r="L24" s="39" t="n"/>
-      <c r="M24" s="40" t="n"/>
+      <c r="D24" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="9" t="n"/>
+      <c r="L24" s="9" t="n"/>
+      <c r="M24" s="9" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1" s="1">
+      <c r="A25" s="26" t="n"/>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>GEÇERLİLİK TARİHİ</t>
+          <t>AKSESUARLAR</t>
         </is>
       </c>
       <c r="C25" s="40" t="n"/>
-      <c r="D25" s="42" t="inlineStr">
-        <is>
-          <t>{gecerlilikTarihi}</t>
-        </is>
-      </c>
-      <c r="E25" s="39" t="n"/>
-      <c r="F25" s="39" t="n"/>
-      <c r="G25" s="39" t="n"/>
-      <c r="H25" s="39" t="n"/>
-      <c r="I25" s="39" t="n"/>
-      <c r="J25" s="39" t="n"/>
-      <c r="K25" s="39" t="n"/>
-      <c r="L25" s="39" t="n"/>
-      <c r="M25" s="40" t="n"/>
+      <c r="D25" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n"/>
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="9" t="n"/>
+      <c r="L25" s="9" t="n"/>
+      <c r="M25" s="9" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1" s="1">
+      <c r="A26" s="26" t="n"/>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>FİYAT LİSTESİ</t>
+          <t>PARKE</t>
         </is>
       </c>
       <c r="C26" s="40" t="n"/>
-      <c r="D26" s="42" t="inlineStr">
-        <is>
-          <t>{fiyatListesiEtiketi} - Para Birimi: {paraBirimi}</t>
-        </is>
-      </c>
-      <c r="E26" s="39" t="n"/>
-      <c r="F26" s="39" t="n"/>
-      <c r="G26" s="39" t="n"/>
-      <c r="H26" s="39" t="n"/>
-      <c r="I26" s="39" t="n"/>
-      <c r="J26" s="39" t="n"/>
-      <c r="K26" s="39" t="n"/>
-      <c r="L26" s="39" t="n"/>
-      <c r="M26" s="40" t="n"/>
+      <c r="D26" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="9" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1" s="1">
       <c r="A27" s="26" t="n"/>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>HİZMETLER &amp; MONTAJ</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="n"/>
+      <c r="D27" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="9" t="n"/>
       <c r="G27" s="9" t="n"/>
@@ -1377,9 +1452,9 @@
     </row>
     <row r="28" ht="24" customHeight="1" s="1">
       <c r="A28" s="26" t="n"/>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>ÜRÜN GRUPLARI</t>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>TOPLAM YEKÜN</t>
         </is>
       </c>
       <c r="C28" s="39" t="n"/>
@@ -1396,11 +1471,7 @@
     </row>
     <row r="29" ht="20" customHeight="1" s="1">
       <c r="A29" s="26" t="n"/>
-      <c r="B29" s="43" t="inlineStr">
-        <is>
-          <t>{urunGruplari}</t>
-        </is>
-      </c>
+      <c r="B29" s="9" t="n"/>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
@@ -1445,118 +1516,119 @@
     </row>
     <row r="32" ht="24" customHeight="1" s="1" thickBot="1">
       <c r="A32" s="26" t="n"/>
-      <c r="B32" s="44" t="inlineStr">
-        <is>
-          <t>YEKÜN İCMAALLERİ</t>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>ÖDEME VE TESLİM</t>
         </is>
       </c>
       <c r="C32" s="39" t="n"/>
       <c r="D32" s="40" t="n"/>
-      <c r="E32" s="9" t="n"/>
-      <c r="F32" s="9" t="n"/>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="9" t="n"/>
-      <c r="I32" s="9" t="n"/>
-      <c r="J32" s="9" t="n"/>
-      <c r="K32" s="9" t="n"/>
-      <c r="L32" s="9" t="n"/>
-      <c r="M32" s="9" t="n"/>
+      <c r="E32" s="39" t="n"/>
+      <c r="F32" s="39" t="n"/>
+      <c r="G32" s="39" t="n"/>
+      <c r="H32" s="39" t="n"/>
+      <c r="I32" s="39" t="n"/>
+      <c r="J32" s="39" t="n"/>
+      <c r="K32" s="39" t="n"/>
+      <c r="L32" s="39" t="n"/>
+      <c r="M32" s="40" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A33" s="26" t="n"/>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>ÇELİK KAPI GRUBU</t>
+          <t>ÖDEME KOŞULU</t>
         </is>
       </c>
       <c r="C33" s="40" t="n"/>
-      <c r="D33" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
-      <c r="I33" s="9" t="n"/>
-      <c r="J33" s="9" t="n"/>
-      <c r="K33" s="9" t="n"/>
-      <c r="L33" s="9" t="n"/>
-      <c r="M33" s="9" t="n"/>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>{odemeKosulu}</t>
+        </is>
+      </c>
+      <c r="E33" s="39" t="n"/>
+      <c r="F33" s="39" t="n"/>
+      <c r="G33" s="39" t="n"/>
+      <c r="H33" s="39" t="n"/>
+      <c r="I33" s="39" t="n"/>
+      <c r="J33" s="39" t="n"/>
+      <c r="K33" s="39" t="n"/>
+      <c r="L33" s="39" t="n"/>
+      <c r="M33" s="40" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A34" s="26" t="n"/>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>İÇ ODA KAPI GRUBU</t>
+          <t>TESLİM TİPİ</t>
         </is>
       </c>
       <c r="C34" s="40" t="n"/>
-      <c r="D34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" s="9" t="n"/>
-      <c r="J34" s="9" t="n"/>
-      <c r="K34" s="9" t="n"/>
-      <c r="L34" s="9" t="n"/>
-      <c r="M34" s="9" t="n"/>
+      <c r="D34" s="42" t="inlineStr">
+        <is>
+          <t>{teslimTipi}</t>
+        </is>
+      </c>
+      <c r="E34" s="39" t="n"/>
+      <c r="F34" s="39" t="n"/>
+      <c r="G34" s="39" t="n"/>
+      <c r="H34" s="39" t="n"/>
+      <c r="I34" s="39" t="n"/>
+      <c r="J34" s="39" t="n"/>
+      <c r="K34" s="39" t="n"/>
+      <c r="L34" s="39" t="n"/>
+      <c r="M34" s="40" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A35" s="26" t="n"/>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>MUTFAK GRUBU</t>
+          <t>TESLİM TARİHİ</t>
         </is>
       </c>
       <c r="C35" s="40" t="n"/>
-      <c r="D35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
-      <c r="I35" s="9" t="n"/>
-      <c r="J35" s="9" t="n"/>
-      <c r="K35" s="9" t="n"/>
-      <c r="L35" s="9" t="n"/>
-      <c r="M35" s="9" t="n"/>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>{teslimTarihi}</t>
+        </is>
+      </c>
+      <c r="E35" s="39" t="n"/>
+      <c r="F35" s="39" t="n"/>
+      <c r="G35" s="39" t="n"/>
+      <c r="H35" s="39" t="n"/>
+      <c r="I35" s="39" t="n"/>
+      <c r="J35" s="39" t="n"/>
+      <c r="K35" s="39" t="n"/>
+      <c r="L35" s="39" t="n"/>
+      <c r="M35" s="40" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A36" s="26" t="n"/>
       <c r="B36" s="22" t="inlineStr">
         <is>
-          <t>PORTMANTO GRUBU</t>
+          <t>NOTLAR</t>
         </is>
       </c>
       <c r="C36" s="40" t="n"/>
-      <c r="D36" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="9" t="n"/>
-      <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="9" t="n"/>
-      <c r="I36" s="9" t="n"/>
-      <c r="J36" s="9" t="n"/>
-      <c r="K36" s="9" t="n"/>
-      <c r="L36" s="9" t="n"/>
-      <c r="M36" s="9" t="n"/>
+      <c r="D36" s="42" t="inlineStr">
+        <is>
+          <t>{notlar}</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="n"/>
+      <c r="F36" s="39" t="n"/>
+      <c r="G36" s="39" t="n"/>
+      <c r="H36" s="39" t="n"/>
+      <c r="I36" s="39" t="n"/>
+      <c r="J36" s="39" t="n"/>
+      <c r="K36" s="39" t="n"/>
+      <c r="L36" s="39" t="n"/>
+      <c r="M36" s="40" t="n"/>
     </row>
     <row r="37" ht="24" customHeight="1" s="1" thickBot="1">
       <c r="A37" s="26" t="n"/>
-      <c r="B37" s="22" t="inlineStr">
-        <is>
-          <t>BANYO DOLAPLARI</t>
-        </is>
-      </c>
-      <c r="C37" s="40" t="n"/>
-      <c r="D37" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="B37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
       <c r="E37" s="9" t="n"/>
       <c r="F37" s="9" t="n"/>
       <c r="G37" s="9" t="n"/>
@@ -1569,15 +1641,8 @@
     </row>
     <row r="38" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A38" s="26" t="n"/>
-      <c r="B38" s="22" t="inlineStr">
-        <is>
-          <t>AKSESUARLAR</t>
-        </is>
-      </c>
-      <c r="C38" s="40" t="n"/>
-      <c r="D38" s="30" t="n">
-        <v>0</v>
-      </c>
+      <c r="B38" s="9" t="n"/>
+      <c r="D38" s="9" t="n"/>
       <c r="E38" s="9" t="n"/>
       <c r="F38" s="9" t="n"/>
       <c r="G38" s="9" t="n"/>
@@ -1590,97 +1655,114 @@
     </row>
     <row r="39" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A39" s="26" t="n"/>
-      <c r="B39" s="22" t="inlineStr">
-        <is>
-          <t>PARKE</t>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>FİRMA ÜNVANI &amp; IBANLAR</t>
         </is>
       </c>
       <c r="C39" s="40" t="n"/>
-      <c r="D39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="9" t="n"/>
-      <c r="F39" s="9" t="n"/>
-      <c r="G39" s="9" t="n"/>
-      <c r="H39" s="9" t="n"/>
-      <c r="I39" s="9" t="n"/>
-      <c r="J39" s="9" t="n"/>
-      <c r="K39" s="9" t="n"/>
-      <c r="L39" s="9" t="n"/>
-      <c r="M39" s="9" t="n"/>
+      <c r="D39" s="39" t="n"/>
+      <c r="E39" s="39" t="n"/>
+      <c r="F39" s="39" t="n"/>
+      <c r="G39" s="39" t="n"/>
+      <c r="H39" s="39" t="n"/>
+      <c r="I39" s="39" t="n"/>
+      <c r="J39" s="39" t="n"/>
+      <c r="K39" s="39" t="n"/>
+      <c r="L39" s="39" t="n"/>
+      <c r="M39" s="40" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1" s="1" thickBot="1">
       <c r="A40" s="26" t="n"/>
       <c r="B40" s="22" t="inlineStr">
         <is>
-          <t>HİZMETLER &amp; MONTAJ</t>
+          <t>{seciliSatici.banka1.ad}</t>
         </is>
       </c>
       <c r="C40" s="40" t="n"/>
-      <c r="D40" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="9" t="n"/>
-      <c r="F40" s="9" t="n"/>
-      <c r="G40" s="9" t="n"/>
-      <c r="H40" s="9" t="n"/>
-      <c r="I40" s="9" t="n"/>
-      <c r="J40" s="9" t="n"/>
-      <c r="K40" s="9" t="n"/>
-      <c r="L40" s="9" t="n"/>
-      <c r="M40" s="9" t="n"/>
+      <c r="D40" s="42" t="inlineStr">
+        <is>
+          <t>{seciliSatici.banka1.iban}</t>
+        </is>
+      </c>
+      <c r="E40" s="39" t="n"/>
+      <c r="F40" s="39" t="n"/>
+      <c r="G40" s="39" t="n"/>
+      <c r="H40" s="39" t="n"/>
+      <c r="I40" s="39" t="n"/>
+      <c r="J40" s="39" t="n"/>
+      <c r="K40" s="39" t="n"/>
+      <c r="L40" s="39" t="n"/>
+      <c r="M40" s="40" t="n"/>
     </row>
     <row r="41" ht="24" customHeight="1" s="1" thickBot="1">
       <c r="A41" s="26" t="n"/>
       <c r="B41" s="22" t="inlineStr">
         <is>
-          <t>TOPLAM YEKÜN</t>
+          <t>{seciliSatici.banka2.ad}</t>
         </is>
       </c>
       <c r="C41" s="40" t="n"/>
-      <c r="D41" s="30">
-        <f>SUM(D33:D40)</f>
-        <v/>
-      </c>
-      <c r="E41" s="9" t="n"/>
-      <c r="F41" s="9" t="n"/>
-      <c r="G41" s="9" t="n"/>
-      <c r="H41" s="9" t="n"/>
-      <c r="I41" s="9" t="n"/>
-      <c r="J41" s="9" t="n"/>
-      <c r="K41" s="9" t="n"/>
-      <c r="L41" s="9" t="n"/>
-      <c r="M41" s="9" t="n"/>
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>{seciliSatici.banka2.iban}</t>
+        </is>
+      </c>
+      <c r="E41" s="39" t="n"/>
+      <c r="F41" s="39" t="n"/>
+      <c r="G41" s="39" t="n"/>
+      <c r="H41" s="39" t="n"/>
+      <c r="I41" s="39" t="n"/>
+      <c r="J41" s="39" t="n"/>
+      <c r="K41" s="39" t="n"/>
+      <c r="L41" s="39" t="n"/>
+      <c r="M41" s="40" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1" s="1">
       <c r="A42" s="26" t="n"/>
-      <c r="B42" s="9" t="n"/>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9" t="n"/>
-      <c r="I42" s="9" t="n"/>
-      <c r="J42" s="9" t="n"/>
-      <c r="K42" s="9" t="n"/>
-      <c r="L42" s="9" t="n"/>
-      <c r="M42" s="9" t="n"/>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>{seciliSatici.banka3.ad}</t>
+        </is>
+      </c>
+      <c r="C42" s="40" t="n"/>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>{seciliSatici.banka3.iban}</t>
+        </is>
+      </c>
+      <c r="E42" s="39" t="n"/>
+      <c r="F42" s="39" t="n"/>
+      <c r="G42" s="39" t="n"/>
+      <c r="H42" s="39" t="n"/>
+      <c r="I42" s="39" t="n"/>
+      <c r="J42" s="39" t="n"/>
+      <c r="K42" s="39" t="n"/>
+      <c r="L42" s="39" t="n"/>
+      <c r="M42" s="40" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1" s="1">
       <c r="A43" s="26" t="n"/>
-      <c r="B43" s="9" t="n"/>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="9" t="n"/>
-      <c r="F43" s="9" t="n"/>
-      <c r="G43" s="9" t="n"/>
-      <c r="H43" s="9" t="n"/>
-      <c r="I43" s="9" t="n"/>
-      <c r="J43" s="9" t="n"/>
-      <c r="K43" s="9" t="n"/>
-      <c r="L43" s="9" t="n"/>
-      <c r="M43" s="9" t="n"/>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>{seciliSatici.banka4.ad}</t>
+        </is>
+      </c>
+      <c r="C43" s="40" t="n"/>
+      <c r="D43" s="42" t="inlineStr">
+        <is>
+          <t>{seciliSatici.banka4.iban}</t>
+        </is>
+      </c>
+      <c r="E43" s="39" t="n"/>
+      <c r="F43" s="39" t="n"/>
+      <c r="G43" s="39" t="n"/>
+      <c r="H43" s="39" t="n"/>
+      <c r="I43" s="39" t="n"/>
+      <c r="J43" s="39" t="n"/>
+      <c r="K43" s="39" t="n"/>
+      <c r="L43" s="39" t="n"/>
+      <c r="M43" s="40" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1" s="1">
       <c r="A44" s="26" t="n"/>
@@ -1699,59 +1781,22 @@
     </row>
     <row r="45" ht="24" customHeight="1" s="1">
       <c r="A45" s="26" t="n"/>
-      <c r="B45" s="15" t="inlineStr">
-        <is>
-          <t>ÖDEME VE TESLİM</t>
-        </is>
-      </c>
-      <c r="C45" s="39" t="n"/>
-      <c r="D45" s="39" t="n"/>
-      <c r="E45" s="39" t="n"/>
-      <c r="F45" s="39" t="n"/>
-      <c r="G45" s="39" t="n"/>
-      <c r="H45" s="39" t="n"/>
-      <c r="I45" s="39" t="n"/>
-      <c r="J45" s="39" t="n"/>
-      <c r="K45" s="39" t="n"/>
-      <c r="L45" s="39" t="n"/>
-      <c r="M45" s="40" t="n"/>
+      <c r="B45" s="9" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1" s="1">
       <c r="A46" s="26" t="n"/>
-      <c r="B46" s="22" t="inlineStr">
-        <is>
-          <t>ÖDEME KOŞULU</t>
-        </is>
-      </c>
-      <c r="C46" s="40" t="n"/>
-      <c r="D46" s="42" t="inlineStr">
-        <is>
-          <t>{odemeKosulu}</t>
-        </is>
-      </c>
-      <c r="E46" s="39" t="n"/>
-      <c r="F46" s="39" t="n"/>
-      <c r="G46" s="39" t="n"/>
-      <c r="H46" s="39" t="n"/>
-      <c r="I46" s="39" t="n"/>
-      <c r="J46" s="39" t="n"/>
-      <c r="K46" s="39" t="n"/>
-      <c r="L46" s="39" t="n"/>
-      <c r="M46" s="40" t="n"/>
+      <c r="B46" s="9" t="n"/>
+      <c r="D46" s="9" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1" s="1">
       <c r="A47" s="26" t="n"/>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>TESLİM TİPİ</t>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>TARAFLARIN KAŞE İMZASI</t>
         </is>
       </c>
       <c r="C47" s="40" t="n"/>
-      <c r="D47" s="42" t="inlineStr">
-        <is>
-          <t>{teslimTipi}</t>
-        </is>
-      </c>
+      <c r="D47" s="40" t="n"/>
       <c r="E47" s="39" t="n"/>
       <c r="F47" s="39" t="n"/>
       <c r="G47" s="39" t="n"/>
@@ -1764,428 +1809,157 @@
     </row>
     <row r="48" ht="20" customHeight="1" s="1">
       <c r="A48" s="26" t="n"/>
-      <c r="B48" s="22" t="inlineStr">
-        <is>
-          <t>TESLİM TARİHİ</t>
+      <c r="B48" s="45" t="inlineStr">
+        <is>
+          <t>SATICI
+{seciliSatici.resmiUnvan}</t>
         </is>
       </c>
       <c r="C48" s="40" t="n"/>
-      <c r="D48" s="42" t="inlineStr">
-        <is>
-          <t>{teslimTarihi}</t>
-        </is>
-      </c>
-      <c r="E48" s="39" t="n"/>
-      <c r="F48" s="39" t="n"/>
-      <c r="G48" s="39" t="n"/>
-      <c r="H48" s="39" t="n"/>
-      <c r="I48" s="39" t="n"/>
-      <c r="J48" s="39" t="n"/>
-      <c r="K48" s="39" t="n"/>
-      <c r="L48" s="39" t="n"/>
-      <c r="M48" s="40" t="n"/>
+      <c r="D48" s="47" t="n"/>
+      <c r="E48" s="46" t="n"/>
+      <c r="F48" s="46" t="n"/>
+      <c r="G48" s="46" t="n"/>
+      <c r="H48" s="46" t="n"/>
+      <c r="I48" s="46" t="n"/>
+      <c r="J48" s="46" t="n"/>
+      <c r="K48" s="46" t="n"/>
+      <c r="L48" s="46" t="n"/>
+      <c r="M48" s="47" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1" s="1">
       <c r="A49" s="26" t="n"/>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>NOTLAR</t>
-        </is>
-      </c>
-      <c r="C49" s="40" t="n"/>
-      <c r="D49" s="42" t="inlineStr">
-        <is>
-          <t>{notlar}</t>
-        </is>
-      </c>
-      <c r="E49" s="39" t="n"/>
-      <c r="F49" s="39" t="n"/>
-      <c r="G49" s="39" t="n"/>
-      <c r="H49" s="39" t="n"/>
-      <c r="I49" s="39" t="n"/>
-      <c r="J49" s="39" t="n"/>
-      <c r="K49" s="39" t="n"/>
-      <c r="L49" s="39" t="n"/>
-      <c r="M49" s="40" t="n"/>
+      <c r="B49" s="48" t="n"/>
+      <c r="D49" s="49" t="n"/>
+      <c r="M49" s="49" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1" s="1">
       <c r="A50" s="26" t="n"/>
-      <c r="B50" s="9" t="n"/>
-      <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="9" t="n"/>
-      <c r="H50" s="9" t="n"/>
-      <c r="I50" s="9" t="n"/>
-      <c r="J50" s="9" t="n"/>
-      <c r="K50" s="9" t="n"/>
-      <c r="L50" s="9" t="n"/>
-      <c r="M50" s="9" t="n"/>
+      <c r="B50" s="48" t="n"/>
+      <c r="G50" s="49" t="n"/>
+      <c r="H50" s="48" t="n"/>
+      <c r="M50" s="49" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1" s="1">
       <c r="A51" s="26" t="n"/>
-      <c r="B51" s="9" t="n"/>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
-      <c r="F51" s="9" t="n"/>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n"/>
-      <c r="I51" s="9" t="n"/>
-      <c r="J51" s="9" t="n"/>
-      <c r="K51" s="9" t="n"/>
-      <c r="L51" s="9" t="n"/>
-      <c r="M51" s="9" t="n"/>
+      <c r="B51" s="48" t="n"/>
+      <c r="G51" s="49" t="n"/>
+      <c r="H51" s="48" t="n"/>
+      <c r="M51" s="49" t="n"/>
     </row>
     <row r="52" ht="24" customHeight="1" s="1">
       <c r="A52" s="26" t="n"/>
-      <c r="B52" s="15" t="inlineStr">
-        <is>
-          <t>FİRMA ÜNVANI &amp; IBANLAR</t>
-        </is>
-      </c>
-      <c r="C52" s="39" t="n"/>
-      <c r="D52" s="39" t="n"/>
-      <c r="E52" s="39" t="n"/>
-      <c r="F52" s="39" t="n"/>
-      <c r="G52" s="39" t="n"/>
-      <c r="H52" s="39" t="n"/>
-      <c r="I52" s="39" t="n"/>
-      <c r="J52" s="39" t="n"/>
-      <c r="K52" s="39" t="n"/>
-      <c r="L52" s="39" t="n"/>
-      <c r="M52" s="40" t="n"/>
+      <c r="B52" s="54" t="n"/>
+      <c r="M52" s="49" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1" s="1">
       <c r="A53" s="26" t="n"/>
-      <c r="B53" s="22" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka1.ad}</t>
-        </is>
-      </c>
-      <c r="C53" s="40" t="n"/>
-      <c r="D53" s="42" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka1.iban}</t>
-        </is>
-      </c>
-      <c r="E53" s="39" t="n"/>
-      <c r="F53" s="39" t="n"/>
-      <c r="G53" s="39" t="n"/>
-      <c r="H53" s="39" t="n"/>
-      <c r="I53" s="39" t="n"/>
-      <c r="J53" s="39" t="n"/>
-      <c r="K53" s="39" t="n"/>
-      <c r="L53" s="39" t="n"/>
-      <c r="M53" s="40" t="n"/>
+      <c r="B53" s="50" t="n"/>
+      <c r="C53" s="51" t="n"/>
+      <c r="D53" s="52" t="n"/>
+      <c r="E53" s="51" t="n"/>
+      <c r="F53" s="51" t="n"/>
+      <c r="G53" s="51" t="n"/>
+      <c r="H53" s="51" t="n"/>
+      <c r="I53" s="51" t="n"/>
+      <c r="J53" s="51" t="n"/>
+      <c r="K53" s="51" t="n"/>
+      <c r="L53" s="51" t="n"/>
+      <c r="M53" s="52" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1" s="1">
       <c r="A54" s="26" t="n"/>
-      <c r="B54" s="22" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka2.ad}</t>
-        </is>
-      </c>
-      <c r="C54" s="40" t="n"/>
-      <c r="D54" s="42" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka2.iban}</t>
-        </is>
-      </c>
-      <c r="E54" s="39" t="n"/>
-      <c r="F54" s="39" t="n"/>
-      <c r="G54" s="39" t="n"/>
-      <c r="H54" s="39" t="n"/>
-      <c r="I54" s="39" t="n"/>
-      <c r="J54" s="39" t="n"/>
-      <c r="K54" s="39" t="n"/>
-      <c r="L54" s="39" t="n"/>
-      <c r="M54" s="40" t="n"/>
+      <c r="B54" s="26" t="n"/>
+      <c r="D54" s="26" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1" s="1">
       <c r="A55" s="26" t="n"/>
-      <c r="B55" s="22" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka3.ad}</t>
-        </is>
-      </c>
-      <c r="C55" s="40" t="n"/>
-      <c r="D55" s="42" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka3.iban}</t>
-        </is>
-      </c>
-      <c r="E55" s="39" t="n"/>
-      <c r="F55" s="39" t="n"/>
-      <c r="G55" s="39" t="n"/>
-      <c r="H55" s="39" t="n"/>
-      <c r="I55" s="39" t="n"/>
-      <c r="J55" s="39" t="n"/>
-      <c r="K55" s="39" t="n"/>
-      <c r="L55" s="39" t="n"/>
-      <c r="M55" s="40" t="n"/>
-    </row>
-    <row r="56" ht="20" customHeight="1" s="1">
-      <c r="A56" s="26" t="n"/>
-      <c r="B56" s="22" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka4.ad}</t>
-        </is>
-      </c>
-      <c r="C56" s="40" t="n"/>
-      <c r="D56" s="42" t="inlineStr">
-        <is>
-          <t>{seciliSatici.banka4.iban}</t>
-        </is>
-      </c>
-      <c r="E56" s="39" t="n"/>
-      <c r="F56" s="39" t="n"/>
-      <c r="G56" s="39" t="n"/>
-      <c r="H56" s="39" t="n"/>
-      <c r="I56" s="39" t="n"/>
-      <c r="J56" s="39" t="n"/>
-      <c r="K56" s="39" t="n"/>
-      <c r="L56" s="39" t="n"/>
-      <c r="M56" s="40" t="n"/>
-    </row>
-    <row r="57" ht="20" customHeight="1" s="1">
-      <c r="A57" s="26" t="n"/>
-      <c r="B57" s="9" t="n"/>
-      <c r="C57" s="9" t="n"/>
-      <c r="D57" s="9" t="n"/>
-      <c r="E57" s="9" t="n"/>
-      <c r="F57" s="9" t="n"/>
-      <c r="G57" s="9" t="n"/>
-      <c r="H57" s="9" t="n"/>
-      <c r="I57" s="9" t="n"/>
-      <c r="J57" s="9" t="n"/>
-      <c r="K57" s="9" t="n"/>
-      <c r="L57" s="9" t="n"/>
-      <c r="M57" s="9" t="n"/>
-    </row>
-    <row r="58" ht="20" customHeight="1" s="1">
-      <c r="A58" s="26" t="n"/>
-      <c r="B58" s="9" t="n"/>
-      <c r="C58" s="9" t="n"/>
-      <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9" t="n"/>
-      <c r="F58" s="9" t="n"/>
-      <c r="G58" s="9" t="n"/>
-      <c r="H58" s="9" t="n"/>
-      <c r="I58" s="9" t="n"/>
-      <c r="J58" s="9" t="n"/>
-      <c r="K58" s="9" t="n"/>
-      <c r="L58" s="9" t="n"/>
-      <c r="M58" s="9" t="n"/>
-    </row>
-    <row r="59" ht="20" customHeight="1" s="1">
-      <c r="A59" s="26" t="n"/>
-      <c r="B59" s="9" t="n"/>
-      <c r="C59" s="9" t="n"/>
-      <c r="D59" s="9" t="n"/>
-      <c r="E59" s="9" t="n"/>
-      <c r="F59" s="9" t="n"/>
-      <c r="G59" s="9" t="n"/>
-      <c r="H59" s="9" t="n"/>
-      <c r="I59" s="9" t="n"/>
-      <c r="J59" s="9" t="n"/>
-      <c r="K59" s="9" t="n"/>
-      <c r="L59" s="9" t="n"/>
-      <c r="M59" s="9" t="n"/>
-    </row>
-    <row r="60" ht="24" customHeight="1" s="1">
-      <c r="A60" s="26" t="n"/>
-      <c r="B60" s="15" t="inlineStr">
-        <is>
-          <t>TARAFLARIN KAŞE İMZASI</t>
-        </is>
-      </c>
-      <c r="C60" s="39" t="n"/>
-      <c r="D60" s="39" t="n"/>
-      <c r="E60" s="39" t="n"/>
-      <c r="F60" s="39" t="n"/>
-      <c r="G60" s="39" t="n"/>
-      <c r="H60" s="39" t="n"/>
-      <c r="I60" s="39" t="n"/>
-      <c r="J60" s="39" t="n"/>
-      <c r="K60" s="39" t="n"/>
-      <c r="L60" s="39" t="n"/>
-      <c r="M60" s="40" t="n"/>
-    </row>
-    <row r="61" ht="20" customHeight="1" s="1">
-      <c r="A61" s="26" t="n"/>
-      <c r="B61" s="45" t="inlineStr">
-        <is>
-          <t>SATICI
-{seciliSatici.resmiUnvan}</t>
-        </is>
-      </c>
-      <c r="C61" s="46" t="n"/>
-      <c r="D61" s="46" t="n"/>
-      <c r="E61" s="46" t="n"/>
-      <c r="F61" s="46" t="n"/>
-      <c r="G61" s="47" t="n"/>
-      <c r="H61" s="45" t="inlineStr">
-        <is>
-          <t>ALICI
-{cariUnvani}</t>
-        </is>
-      </c>
-      <c r="I61" s="46" t="n"/>
-      <c r="J61" s="46" t="n"/>
-      <c r="K61" s="46" t="n"/>
-      <c r="L61" s="46" t="n"/>
-      <c r="M61" s="47" t="n"/>
-    </row>
-    <row r="62" ht="20" customHeight="1" s="1">
-      <c r="A62" s="26" t="n"/>
-      <c r="B62" s="48" t="n"/>
-      <c r="G62" s="49" t="n"/>
-      <c r="H62" s="48" t="n"/>
-      <c r="M62" s="49" t="n"/>
-    </row>
-    <row r="63" ht="20" customHeight="1" s="1">
-      <c r="A63" s="26" t="n"/>
-      <c r="B63" s="48" t="n"/>
-      <c r="G63" s="49" t="n"/>
-      <c r="H63" s="48" t="n"/>
-      <c r="M63" s="49" t="n"/>
-    </row>
-    <row r="64" ht="20" customHeight="1" s="1">
-      <c r="A64" s="26" t="n"/>
-      <c r="B64" s="48" t="n"/>
-      <c r="G64" s="49" t="n"/>
-      <c r="H64" s="48" t="n"/>
-      <c r="M64" s="49" t="n"/>
-    </row>
-    <row r="65" ht="20" customHeight="1" s="1">
-      <c r="A65" s="26" t="n"/>
-      <c r="B65" s="48" t="n"/>
-      <c r="G65" s="49" t="n"/>
-      <c r="H65" s="48" t="n"/>
-      <c r="M65" s="49" t="n"/>
-    </row>
-    <row r="66" ht="20" customHeight="1" s="1">
-      <c r="A66" s="26" t="n"/>
-      <c r="B66" s="50" t="n"/>
-      <c r="C66" s="51" t="n"/>
-      <c r="D66" s="51" t="n"/>
-      <c r="E66" s="51" t="n"/>
-      <c r="F66" s="51" t="n"/>
-      <c r="G66" s="52" t="n"/>
-      <c r="H66" s="50" t="n"/>
-      <c r="I66" s="51" t="n"/>
-      <c r="J66" s="51" t="n"/>
-      <c r="K66" s="51" t="n"/>
-      <c r="L66" s="51" t="n"/>
-      <c r="M66" s="52" t="n"/>
-    </row>
-    <row r="67" ht="20" customHeight="1" s="1">
-      <c r="A67" s="26" t="n"/>
-      <c r="B67" s="26" t="n"/>
-      <c r="C67" s="26" t="n"/>
-      <c r="D67" s="26" t="n"/>
-      <c r="E67" s="26" t="n"/>
-      <c r="F67" s="26" t="n"/>
-      <c r="G67" s="26" t="n"/>
-      <c r="H67" s="26" t="n"/>
-      <c r="I67" s="26" t="n"/>
-      <c r="J67" s="26" t="n"/>
-      <c r="K67" s="26" t="n"/>
-      <c r="L67" s="26" t="n"/>
-      <c r="M67" s="26" t="n"/>
-    </row>
-    <row r="68" ht="20" customHeight="1" s="1">
-      <c r="A68" s="26" t="n"/>
-      <c r="B68" s="26" t="n"/>
-      <c r="C68" s="26" t="n"/>
-      <c r="D68" s="26" t="n"/>
-      <c r="E68" s="26" t="n"/>
-      <c r="F68" s="26" t="n"/>
-      <c r="G68" s="26" t="n"/>
-      <c r="H68" s="26" t="n"/>
-      <c r="I68" s="26" t="n"/>
-      <c r="J68" s="26" t="n"/>
-      <c r="K68" s="26" t="n"/>
-      <c r="L68" s="26" t="n"/>
-      <c r="M68" s="26" t="n"/>
-    </row>
+      <c r="B55" s="26" t="n"/>
+      <c r="D55" s="26" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1" s="1"/>
+    <row r="57" ht="20" customHeight="1" s="1"/>
+    <row r="58" ht="20" customHeight="1" s="1"/>
+    <row r="59" ht="20" customHeight="1" s="1"/>
+    <row r="60" ht="24" customHeight="1" s="1"/>
+    <row r="61" ht="20" customHeight="1" s="1"/>
+    <row r="62" ht="20" customHeight="1" s="1"/>
+    <row r="63" ht="20" customHeight="1" s="1"/>
+    <row r="64" ht="20" customHeight="1" s="1"/>
+    <row r="65" ht="20" customHeight="1" s="1"/>
+    <row r="66" ht="20" customHeight="1" s="1"/>
+    <row r="67" ht="20" customHeight="1" s="1"/>
+    <row r="68" ht="20" customHeight="1" s="1"/>
     <row r="69" ht="20" customHeight="1" s="1"/>
   </sheetData>
-  <mergeCells count="69">
+  <mergeCells count="63">
     <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="B60:M60"/>
+    <mergeCell ref="H10:I10"/>
     <mergeCell ref="D56:M56"/>
-    <mergeCell ref="B60:M60"/>
-    <mergeCell ref="M8"/>
-    <mergeCell ref="D12:M12"/>
-    <mergeCell ref="D18:M18"/>
     <mergeCell ref="B46:C46"/>
-    <mergeCell ref="D25:M25"/>
+    <mergeCell ref="J12:M12"/>
+    <mergeCell ref="J2:M2"/>
     <mergeCell ref="B2:E5"/>
     <mergeCell ref="B56:C56"/>
     <mergeCell ref="D55:M55"/>
-    <mergeCell ref="D24:M24"/>
-    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D14:G14"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D23:M23"/>
+    <mergeCell ref="L3:M3"/>
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="B28:M28"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D54:M54"/>
-    <mergeCell ref="D26:M26"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D20:M20"/>
-    <mergeCell ref="B9:M9"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D10:M10"/>
-    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="D10:G10"/>
     <mergeCell ref="B53:C53"/>
-    <mergeCell ref="D19:M19"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="H11:I11"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B15:M15"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="L4:M4"/>
     <mergeCell ref="D46:M46"/>
-    <mergeCell ref="A9:A26"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="B45:M45"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B37:C37"/>
     <mergeCell ref="B61:G66"/>
+    <mergeCell ref="D13:G13"/>
     <mergeCell ref="B40:C40"/>
-    <mergeCell ref="J2:M3"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="H13:I13"/>
     <mergeCell ref="B49:C49"/>
-    <mergeCell ref="D13:M13"/>
     <mergeCell ref="D49:M49"/>
-    <mergeCell ref="D11:M11"/>
     <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="H12:I12"/>
     <mergeCell ref="B7:M7"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D17:M17"/>
-    <mergeCell ref="J4:M4"/>
     <mergeCell ref="D48:M48"/>
-    <mergeCell ref="B22:M22"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="H9:M9"/>
     <mergeCell ref="D53:M53"/>
+    <mergeCell ref="H61:M66"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="H61:M66"/>
     <mergeCell ref="D47:M47"/>
-    <mergeCell ref="D16:M16"/>
-    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="H14:I14"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B52:M52"/>
     <mergeCell ref="B35:C35"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>